<commit_message>
after gust and ry rx corrections
</commit_message>
<xml_diff>
--- a/output/2024-04-01.xlsx
+++ b/output/2024-04-01.xlsx
@@ -628,25 +628,25 @@
         <v>5.23</v>
       </c>
       <c r="F14" t="n">
-        <v>12.96</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>174.8</v>
+        <v>198.9</v>
       </c>
       <c r="H14" t="n">
-        <v>85.7</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="I14" t="n">
         <v>16</v>
       </c>
       <c r="J14" t="n">
-        <v>-24.82</v>
+        <v>-29.03</v>
       </c>
       <c r="K14" t="n">
-        <v>-59.45</v>
+        <v>-64.43000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>64.42</v>
+        <v>70.66</v>
       </c>
     </row>
     <row r="15">
@@ -670,25 +670,25 @@
         <v>5.21</v>
       </c>
       <c r="F15" t="n">
-        <v>12.14</v>
+        <v>13.63</v>
       </c>
       <c r="G15" t="n">
-        <v>190.8</v>
+        <v>182.5</v>
       </c>
       <c r="H15" t="n">
-        <v>87</v>
+        <v>93.2</v>
       </c>
       <c r="I15" t="n">
         <v>16</v>
       </c>
       <c r="J15" t="n">
-        <v>-30.26</v>
+        <v>-37.36</v>
       </c>
       <c r="K15" t="n">
-        <v>53.17</v>
+        <v>60.78</v>
       </c>
       <c r="L15" t="n">
-        <v>61.18</v>
+        <v>71.34</v>
       </c>
     </row>
     <row r="16">
@@ -712,25 +712,25 @@
         <v>5.2</v>
       </c>
       <c r="F16" t="n">
-        <v>12.28</v>
+        <v>12.53</v>
       </c>
       <c r="G16" t="n">
-        <v>169.3</v>
+        <v>185.3</v>
       </c>
       <c r="H16" t="n">
-        <v>93.2</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="I16" t="n">
         <v>16</v>
       </c>
       <c r="J16" t="n">
-        <v>-77</v>
+        <v>-82.02</v>
       </c>
       <c r="K16" t="n">
-        <v>-58.2</v>
+        <v>-63.26</v>
       </c>
       <c r="L16" t="n">
-        <v>96.52</v>
+        <v>103.59</v>
       </c>
     </row>
     <row r="17">
@@ -754,25 +754,25 @@
         <v>4.54</v>
       </c>
       <c r="F17" t="n">
-        <v>12.17</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="G17" t="n">
-        <v>181.8</v>
+        <v>183.1</v>
       </c>
       <c r="H17" t="n">
-        <v>90.7</v>
+        <v>88.7</v>
       </c>
       <c r="I17" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J17" t="n">
-        <v>41.64</v>
+        <v>41.86</v>
       </c>
       <c r="K17" t="n">
-        <v>99.48999999999999</v>
+        <v>96.31</v>
       </c>
       <c r="L17" t="n">
-        <v>107.85</v>
+        <v>105.02</v>
       </c>
     </row>
     <row r="18">
@@ -796,25 +796,25 @@
         <v>4.63</v>
       </c>
       <c r="F18" t="n">
-        <v>12.37</v>
+        <v>10.07</v>
       </c>
       <c r="G18" t="n">
-        <v>187.6</v>
+        <v>187.1</v>
       </c>
       <c r="H18" t="n">
-        <v>89.7</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J18" t="n">
-        <v>16.86</v>
+        <v>15.27</v>
       </c>
       <c r="K18" t="n">
-        <v>34.91</v>
+        <v>22.72</v>
       </c>
       <c r="L18" t="n">
-        <v>38.77</v>
+        <v>27.38</v>
       </c>
     </row>
     <row r="19">
@@ -838,25 +838,25 @@
         <v>5.69</v>
       </c>
       <c r="F19" t="n">
-        <v>12.06</v>
+        <v>11.58</v>
       </c>
       <c r="G19" t="n">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="H19" t="n">
-        <v>89.5</v>
+        <v>84.7</v>
       </c>
       <c r="I19" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J19" t="n">
-        <v>100.79</v>
+        <v>98.97</v>
       </c>
       <c r="K19" t="n">
-        <v>-66.36</v>
+        <v>-71.65000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>120.68</v>
+        <v>122.18</v>
       </c>
     </row>
     <row r="20">
@@ -880,25 +880,25 @@
         <v>4.47</v>
       </c>
       <c r="F20" t="n">
-        <v>12.09</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="G20" t="n">
-        <v>177.2</v>
+        <v>181.5</v>
       </c>
       <c r="H20" t="n">
-        <v>89.90000000000001</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="I20" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J20" t="n">
-        <v>141.51</v>
+        <v>150.09</v>
       </c>
       <c r="K20" t="n">
-        <v>-25.59</v>
+        <v>-49.63</v>
       </c>
       <c r="L20" t="n">
-        <v>143.81</v>
+        <v>158.08</v>
       </c>
     </row>
     <row r="21">
@@ -922,25 +922,25 @@
         <v>4.05</v>
       </c>
       <c r="F21" t="n">
-        <v>13.03</v>
+        <v>12.21</v>
       </c>
       <c r="G21" t="n">
-        <v>176.9</v>
+        <v>200.4</v>
       </c>
       <c r="H21" t="n">
-        <v>85.5</v>
+        <v>86.2</v>
       </c>
       <c r="I21" t="n">
         <v>16</v>
       </c>
       <c r="J21" t="n">
-        <v>-136.74</v>
+        <v>-159.42</v>
       </c>
       <c r="K21" t="n">
-        <v>-54.85</v>
+        <v>-76.23999999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>147.33</v>
+        <v>176.72</v>
       </c>
     </row>
     <row r="22">
@@ -964,25 +964,25 @@
         <v>4.89</v>
       </c>
       <c r="F22" t="n">
-        <v>12.61</v>
+        <v>9.67</v>
       </c>
       <c r="G22" t="n">
-        <v>183.7</v>
+        <v>191.9</v>
       </c>
       <c r="H22" t="n">
-        <v>86.7</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="I22" t="n">
         <v>16</v>
       </c>
       <c r="J22" t="n">
-        <v>-101.54</v>
+        <v>-101.13</v>
       </c>
       <c r="K22" t="n">
-        <v>-67.16</v>
+        <v>-98.84</v>
       </c>
       <c r="L22" t="n">
-        <v>121.75</v>
+        <v>141.41</v>
       </c>
     </row>
     <row r="23">
@@ -1006,25 +1006,25 @@
         <v>4.58</v>
       </c>
       <c r="F23" t="n">
-        <v>12.71</v>
+        <v>10.75</v>
       </c>
       <c r="G23" t="n">
-        <v>189.5</v>
+        <v>193.8</v>
       </c>
       <c r="H23" t="n">
-        <v>88.40000000000001</v>
+        <v>92.5</v>
       </c>
       <c r="I23" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J23" t="n">
-        <v>135.51</v>
+        <v>99.72</v>
       </c>
       <c r="K23" t="n">
-        <v>-47.55</v>
+        <v>-130.44</v>
       </c>
       <c r="L23" t="n">
-        <v>143.61</v>
+        <v>164.19</v>
       </c>
     </row>
     <row r="24">
@@ -1048,25 +1048,25 @@
         <v>4.8</v>
       </c>
       <c r="F24" t="n">
-        <v>13.14</v>
+        <v>11.4</v>
       </c>
       <c r="G24" t="n">
-        <v>184.9</v>
+        <v>202.4</v>
       </c>
       <c r="H24" t="n">
-        <v>91.90000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="I24" t="n">
         <v>16</v>
       </c>
       <c r="J24" t="n">
-        <v>74.58</v>
+        <v>47.06</v>
       </c>
       <c r="K24" t="n">
-        <v>-189.03</v>
+        <v>-228.42</v>
       </c>
       <c r="L24" t="n">
-        <v>203.21</v>
+        <v>233.21</v>
       </c>
     </row>
     <row r="25">
@@ -1090,25 +1090,25 @@
         <v>4.37</v>
       </c>
       <c r="F25" t="n">
-        <v>12.67</v>
+        <v>10.35</v>
       </c>
       <c r="G25" t="n">
-        <v>171.7</v>
+        <v>193.1</v>
       </c>
       <c r="H25" t="n">
-        <v>92.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="I25" t="n">
         <v>16</v>
       </c>
       <c r="J25" t="n">
-        <v>-174.69</v>
+        <v>-187.78</v>
       </c>
       <c r="K25" t="n">
-        <v>-101.42</v>
+        <v>-134.63</v>
       </c>
       <c r="L25" t="n">
-        <v>201.99</v>
+        <v>231.05</v>
       </c>
     </row>
     <row r="26">
@@ -1132,25 +1132,25 @@
         <v>4.93</v>
       </c>
       <c r="F26" t="n">
-        <v>12.2</v>
+        <v>10.86</v>
       </c>
       <c r="G26" t="n">
-        <v>184.9</v>
+        <v>183.7</v>
       </c>
       <c r="H26" t="n">
-        <v>89.40000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="I26" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J26" t="n">
-        <v>277.5</v>
+        <v>263.38</v>
       </c>
       <c r="K26" t="n">
-        <v>-537.2</v>
+        <v>-540.3200000000001</v>
       </c>
       <c r="L26" t="n">
-        <v>604.64</v>
+        <v>601.1</v>
       </c>
     </row>
     <row r="27">
@@ -1174,25 +1174,25 @@
         <v>4.74</v>
       </c>
       <c r="F27" t="n">
-        <v>12.43</v>
+        <v>11.29</v>
       </c>
       <c r="G27" t="n">
-        <v>171.6</v>
+        <v>188.3</v>
       </c>
       <c r="H27" t="n">
-        <v>89.09999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="I27" t="n">
         <v>16</v>
       </c>
       <c r="J27" t="n">
-        <v>-362.23</v>
+        <v>-405.39</v>
       </c>
       <c r="K27" t="n">
-        <v>152.88</v>
+        <v>119.21</v>
       </c>
       <c r="L27" t="n">
-        <v>393.17</v>
+        <v>422.56</v>
       </c>
     </row>
     <row r="28">
@@ -1216,25 +1216,25 @@
         <v>4.71</v>
       </c>
       <c r="F28" t="n">
-        <v>12.82</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="G28" t="n">
-        <v>183</v>
+        <v>196.1</v>
       </c>
       <c r="H28" t="n">
-        <v>86.40000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="I28" t="n">
         <v>16</v>
       </c>
       <c r="J28" t="n">
-        <v>374.26</v>
+        <v>378.9</v>
       </c>
       <c r="K28" t="n">
-        <v>205.79</v>
+        <v>185.34</v>
       </c>
       <c r="L28" t="n">
-        <v>427.11</v>
+        <v>421.81</v>
       </c>
     </row>
     <row r="29">
@@ -1258,25 +1258,25 @@
         <v>5.06</v>
       </c>
       <c r="F29" t="n">
-        <v>12.33</v>
+        <v>12.31</v>
       </c>
       <c r="G29" t="n">
-        <v>183.3</v>
+        <v>186.2</v>
       </c>
       <c r="H29" t="n">
-        <v>93.90000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="I29" t="n">
         <v>16</v>
       </c>
       <c r="J29" t="n">
-        <v>60.12</v>
+        <v>63.85</v>
       </c>
       <c r="K29" t="n">
-        <v>-74.01000000000001</v>
+        <v>-80.78</v>
       </c>
       <c r="L29" t="n">
-        <v>95.34999999999999</v>
+        <v>102.97</v>
       </c>
     </row>
     <row r="30">
@@ -1300,25 +1300,25 @@
         <v>5.21</v>
       </c>
       <c r="F30" t="n">
-        <v>12.6</v>
+        <v>12.14</v>
       </c>
       <c r="G30" t="n">
-        <v>195.1</v>
+        <v>191.7</v>
       </c>
       <c r="H30" t="n">
-        <v>90.90000000000001</v>
+        <v>95.3</v>
       </c>
       <c r="I30" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J30" t="n">
-        <v>40.7</v>
+        <v>42.26</v>
       </c>
       <c r="K30" t="n">
-        <v>-90.86</v>
+        <v>-96.51000000000001</v>
       </c>
       <c r="L30" t="n">
-        <v>99.56</v>
+        <v>105.36</v>
       </c>
     </row>
     <row r="31">
@@ -1342,25 +1342,25 @@
         <v>4.88</v>
       </c>
       <c r="F31" t="n">
-        <v>12.02</v>
+        <v>10.55</v>
       </c>
       <c r="G31" t="n">
-        <v>190.8</v>
+        <v>180.1</v>
       </c>
       <c r="H31" t="n">
-        <v>96.59999999999999</v>
+        <v>93.2</v>
       </c>
       <c r="I31" t="n">
         <v>16</v>
       </c>
       <c r="J31" t="n">
-        <v>1.79</v>
+        <v>2.35</v>
       </c>
       <c r="K31" t="n">
-        <v>-85.89</v>
+        <v>-91.91</v>
       </c>
       <c r="L31" t="n">
-        <v>85.91</v>
+        <v>91.94</v>
       </c>
     </row>
     <row r="32">
@@ -1384,25 +1384,25 @@
         <v>4.67</v>
       </c>
       <c r="F32" t="n">
-        <v>12.54</v>
+        <v>9.91</v>
       </c>
       <c r="G32" t="n">
-        <v>194.9</v>
+        <v>190.6</v>
       </c>
       <c r="H32" t="n">
-        <v>88</v>
+        <v>95.2</v>
       </c>
       <c r="I32" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J32" t="n">
-        <v>66.25</v>
+        <v>75.55</v>
       </c>
       <c r="K32" t="n">
-        <v>3.77</v>
+        <v>-11.4</v>
       </c>
       <c r="L32" t="n">
-        <v>66.34999999999999</v>
+        <v>76.41</v>
       </c>
     </row>
     <row r="33">
@@ -1426,25 +1426,25 @@
         <v>5.11</v>
       </c>
       <c r="F33" t="n">
-        <v>11.67</v>
+        <v>8.92</v>
       </c>
       <c r="G33" t="n">
-        <v>190.4</v>
+        <v>173</v>
       </c>
       <c r="H33" t="n">
-        <v>88.2</v>
+        <v>93</v>
       </c>
       <c r="I33" t="n">
         <v>16</v>
       </c>
       <c r="J33" t="n">
-        <v>37.6</v>
+        <v>44.15</v>
       </c>
       <c r="K33" t="n">
-        <v>82.64</v>
+        <v>82.78</v>
       </c>
       <c r="L33" t="n">
-        <v>90.79000000000001</v>
+        <v>93.81999999999999</v>
       </c>
     </row>
     <row r="34">
@@ -1468,25 +1468,25 @@
         <v>4.73</v>
       </c>
       <c r="F34" t="n">
-        <v>12.39</v>
+        <v>12.54</v>
       </c>
       <c r="G34" t="n">
         <v>187.6</v>
       </c>
       <c r="H34" t="n">
-        <v>94.90000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="I34" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J34" t="n">
-        <v>-86.54000000000001</v>
+        <v>-93.38</v>
       </c>
       <c r="K34" t="n">
-        <v>-20.39</v>
+        <v>-28.12</v>
       </c>
       <c r="L34" t="n">
-        <v>88.91</v>
+        <v>97.52</v>
       </c>
     </row>
     <row r="35">
@@ -1513,22 +1513,22 @@
         <v>12.89</v>
       </c>
       <c r="G35" t="n">
-        <v>184.7</v>
+        <v>197.6</v>
       </c>
       <c r="H35" t="n">
-        <v>86.40000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="I35" t="n">
         <v>16</v>
       </c>
       <c r="J35" t="n">
-        <v>-139.35</v>
+        <v>-163.23</v>
       </c>
       <c r="K35" t="n">
-        <v>13.71</v>
+        <v>-15.31</v>
       </c>
       <c r="L35" t="n">
-        <v>140.02</v>
+        <v>163.95</v>
       </c>
     </row>
     <row r="36">
@@ -1552,25 +1552,25 @@
         <v>5.32</v>
       </c>
       <c r="F36" t="n">
-        <v>12.64</v>
+        <v>14.14</v>
       </c>
       <c r="G36" t="n">
-        <v>192.6</v>
+        <v>192.4</v>
       </c>
       <c r="H36" t="n">
-        <v>95.90000000000001</v>
+        <v>94</v>
       </c>
       <c r="I36" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J36" t="n">
-        <v>224.92</v>
+        <v>251.35</v>
       </c>
       <c r="K36" t="n">
-        <v>-32.57</v>
+        <v>-58.45</v>
       </c>
       <c r="L36" t="n">
-        <v>227.27</v>
+        <v>258.05</v>
       </c>
     </row>
     <row r="37">
@@ -1594,25 +1594,25 @@
         <v>4.21</v>
       </c>
       <c r="F37" t="n">
-        <v>11.66</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G37" t="n">
-        <v>196.2</v>
+        <v>172.9</v>
       </c>
       <c r="H37" t="n">
-        <v>91</v>
+        <v>95.8</v>
       </c>
       <c r="I37" t="n">
         <v>16</v>
       </c>
       <c r="J37" t="n">
-        <v>-156.68</v>
+        <v>-157.58</v>
       </c>
       <c r="K37" t="n">
-        <v>-85.89</v>
+        <v>-105.56</v>
       </c>
       <c r="L37" t="n">
-        <v>178.68</v>
+        <v>189.67</v>
       </c>
     </row>
     <row r="38">
@@ -1636,25 +1636,25 @@
         <v>5.19</v>
       </c>
       <c r="F38" t="n">
-        <v>11.38</v>
+        <v>12.58</v>
       </c>
       <c r="G38" t="n">
-        <v>174.4</v>
+        <v>167.2</v>
       </c>
       <c r="H38" t="n">
-        <v>91.7</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="I38" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J38" t="n">
-        <v>-153.76</v>
+        <v>-190.82</v>
       </c>
       <c r="K38" t="n">
-        <v>91.18000000000001</v>
+        <v>34.52</v>
       </c>
       <c r="L38" t="n">
-        <v>178.76</v>
+        <v>193.91</v>
       </c>
     </row>
     <row r="39">
@@ -1678,25 +1678,25 @@
         <v>5.3</v>
       </c>
       <c r="F39" t="n">
-        <v>12.39</v>
+        <v>11.51</v>
       </c>
       <c r="G39" t="n">
-        <v>191.8</v>
+        <v>187.5</v>
       </c>
       <c r="H39" t="n">
-        <v>91.2</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="I39" t="n">
         <v>16</v>
       </c>
       <c r="J39" t="n">
-        <v>-189.94</v>
+        <v>-191.72</v>
       </c>
       <c r="K39" t="n">
-        <v>-94.67</v>
+        <v>-145.95</v>
       </c>
       <c r="L39" t="n">
-        <v>212.22</v>
+        <v>240.95</v>
       </c>
     </row>
     <row r="40">
@@ -1720,25 +1720,25 @@
         <v>5.11</v>
       </c>
       <c r="F40" t="n">
-        <v>12.19</v>
+        <v>11.46</v>
       </c>
       <c r="G40" t="n">
-        <v>189.9</v>
+        <v>183.6</v>
       </c>
       <c r="H40" t="n">
-        <v>89</v>
+        <v>92.7</v>
       </c>
       <c r="I40" t="n">
         <v>17</v>
       </c>
       <c r="J40" t="n">
-        <v>120.46</v>
+        <v>122.2</v>
       </c>
       <c r="K40" t="n">
-        <v>-329.29</v>
+        <v>-363.42</v>
       </c>
       <c r="L40" t="n">
-        <v>350.63</v>
+        <v>383.42</v>
       </c>
     </row>
     <row r="41">
@@ -1762,25 +1762,25 @@
         <v>4.56</v>
       </c>
       <c r="F41" t="n">
-        <v>12.19</v>
+        <v>7.43</v>
       </c>
       <c r="G41" t="n">
-        <v>191.7</v>
+        <v>183.4</v>
       </c>
       <c r="H41" t="n">
-        <v>87.90000000000001</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="I41" t="n">
         <v>16</v>
       </c>
       <c r="J41" t="n">
-        <v>241.84</v>
+        <v>260.71</v>
       </c>
       <c r="K41" t="n">
-        <v>256.71</v>
+        <v>227.17</v>
       </c>
       <c r="L41" t="n">
-        <v>352.68</v>
+        <v>345.8</v>
       </c>
     </row>
     <row r="42">
@@ -1804,25 +1804,25 @@
         <v>5.05</v>
       </c>
       <c r="F42" t="n">
-        <v>12.34</v>
+        <v>11.8</v>
       </c>
       <c r="G42" t="n">
-        <v>196.5</v>
+        <v>186.4</v>
       </c>
       <c r="H42" t="n">
-        <v>90.2</v>
+        <v>96</v>
       </c>
       <c r="I42" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J42" t="n">
-        <v>-155.81</v>
+        <v>-159.67</v>
       </c>
       <c r="K42" t="n">
-        <v>-402.73</v>
+        <v>-469.29</v>
       </c>
       <c r="L42" t="n">
-        <v>431.81</v>
+        <v>495.71</v>
       </c>
     </row>
     <row r="43">
@@ -1846,25 +1846,25 @@
         <v>4.73</v>
       </c>
       <c r="F43" t="n">
-        <v>12.46</v>
+        <v>12.35</v>
       </c>
       <c r="G43" t="n">
-        <v>174.6</v>
+        <v>188.8</v>
       </c>
       <c r="H43" t="n">
-        <v>97.5</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="I43" t="n">
         <v>16</v>
       </c>
       <c r="J43" t="n">
-        <v>218.77</v>
+        <v>192.62</v>
       </c>
       <c r="K43" t="n">
-        <v>-159.88</v>
+        <v>-245.2</v>
       </c>
       <c r="L43" t="n">
-        <v>270.96</v>
+        <v>311.81</v>
       </c>
     </row>
     <row r="44">
@@ -1888,25 +1888,25 @@
         <v>4.42</v>
       </c>
       <c r="F44" t="n">
-        <v>11.87</v>
+        <v>9.68</v>
       </c>
       <c r="G44" t="n">
-        <v>181.4</v>
+        <v>177.1</v>
       </c>
       <c r="H44" t="n">
-        <v>88.2</v>
+        <v>88.5</v>
       </c>
       <c r="I44" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J44" t="n">
-        <v>53.17</v>
+        <v>56.24</v>
       </c>
       <c r="K44" t="n">
-        <v>-27.62</v>
+        <v>-32.12</v>
       </c>
       <c r="L44" t="n">
-        <v>59.92</v>
+        <v>64.77</v>
       </c>
     </row>
     <row r="45">
@@ -1930,25 +1930,25 @@
         <v>5.28</v>
       </c>
       <c r="F45" t="n">
-        <v>12.73</v>
+        <v>14.14</v>
       </c>
       <c r="G45" t="n">
-        <v>173.9</v>
+        <v>194.2</v>
       </c>
       <c r="H45" t="n">
-        <v>89.2</v>
+        <v>84.7</v>
       </c>
       <c r="I45" t="n">
         <v>16</v>
       </c>
       <c r="J45" t="n">
-        <v>79.44</v>
+        <v>88.28</v>
       </c>
       <c r="K45" t="n">
-        <v>24.47</v>
+        <v>25.53</v>
       </c>
       <c r="L45" t="n">
-        <v>83.12</v>
+        <v>91.90000000000001</v>
       </c>
     </row>
     <row r="46">
@@ -1972,25 +1972,25 @@
         <v>5.1</v>
       </c>
       <c r="F46" t="n">
-        <v>12.33</v>
+        <v>14.14</v>
       </c>
       <c r="G46" t="n">
-        <v>202.3</v>
+        <v>186.3</v>
       </c>
       <c r="H46" t="n">
-        <v>98.40000000000001</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="I46" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J46" t="n">
-        <v>65.34</v>
+        <v>77.02</v>
       </c>
       <c r="K46" t="n">
-        <v>-54.17</v>
+        <v>-65.62</v>
       </c>
       <c r="L46" t="n">
-        <v>84.87</v>
+        <v>101.18</v>
       </c>
     </row>
     <row r="47">
@@ -2014,25 +2014,25 @@
         <v>5.31</v>
       </c>
       <c r="F47" t="n">
-        <v>11.47</v>
+        <v>13.19</v>
       </c>
       <c r="G47" t="n">
-        <v>173</v>
+        <v>169.1</v>
       </c>
       <c r="H47" t="n">
-        <v>87.3</v>
+        <v>84.2</v>
       </c>
       <c r="I47" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J47" t="n">
-        <v>-59.9</v>
+        <v>-66.08</v>
       </c>
       <c r="K47" t="n">
-        <v>-47.59</v>
+        <v>-64.54000000000001</v>
       </c>
       <c r="L47" t="n">
-        <v>76.51000000000001</v>
+        <v>92.37</v>
       </c>
     </row>
     <row r="48">
@@ -2056,25 +2056,25 @@
         <v>5.95</v>
       </c>
       <c r="F48" t="n">
-        <v>12.14</v>
+        <v>12.91</v>
       </c>
       <c r="G48" t="n">
-        <v>188.5</v>
+        <v>182.4</v>
       </c>
       <c r="H48" t="n">
-        <v>86.8</v>
+        <v>92</v>
       </c>
       <c r="I48" t="n">
         <v>16</v>
       </c>
       <c r="J48" t="n">
-        <v>26.7</v>
+        <v>33.83</v>
       </c>
       <c r="K48" t="n">
-        <v>83.65000000000001</v>
+        <v>88.88</v>
       </c>
       <c r="L48" t="n">
-        <v>87.8</v>
+        <v>95.09999999999999</v>
       </c>
     </row>
     <row r="49">
@@ -2098,25 +2098,25 @@
         <v>5.06</v>
       </c>
       <c r="F49" t="n">
-        <v>12.39</v>
+        <v>10.52</v>
       </c>
       <c r="G49" t="n">
-        <v>206.5</v>
+        <v>187.5</v>
       </c>
       <c r="H49" t="n">
-        <v>90.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="I49" t="n">
         <v>16</v>
       </c>
       <c r="J49" t="n">
-        <v>9.41</v>
+        <v>13.76</v>
       </c>
       <c r="K49" t="n">
-        <v>77.55</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="L49" t="n">
-        <v>78.12</v>
+        <v>84.66</v>
       </c>
     </row>
     <row r="50">
@@ -2140,25 +2140,25 @@
         <v>5.2</v>
       </c>
       <c r="F50" t="n">
-        <v>11.96</v>
+        <v>11.41</v>
       </c>
       <c r="G50" t="n">
-        <v>189.1</v>
+        <v>178.9</v>
       </c>
       <c r="H50" t="n">
-        <v>87.5</v>
+        <v>92.3</v>
       </c>
       <c r="I50" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J50" t="n">
-        <v>106</v>
+        <v>130.92</v>
       </c>
       <c r="K50" t="n">
-        <v>96.5</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="L50" t="n">
-        <v>143.35</v>
+        <v>149.97</v>
       </c>
     </row>
     <row r="51">
@@ -2182,25 +2182,25 @@
         <v>5.65</v>
       </c>
       <c r="F51" t="n">
-        <v>12.67</v>
+        <v>13.22</v>
       </c>
       <c r="G51" t="n">
-        <v>183.2</v>
+        <v>193.2</v>
       </c>
       <c r="H51" t="n">
-        <v>92.40000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="I51" t="n">
         <v>16</v>
       </c>
       <c r="J51" t="n">
-        <v>-37.86</v>
+        <v>-45.93</v>
       </c>
       <c r="K51" t="n">
-        <v>-234.83</v>
+        <v>-257.81</v>
       </c>
       <c r="L51" t="n">
-        <v>237.87</v>
+        <v>261.87</v>
       </c>
     </row>
     <row r="52">
@@ -2224,25 +2224,25 @@
         <v>4.64</v>
       </c>
       <c r="F52" t="n">
-        <v>11.7</v>
+        <v>12.48</v>
       </c>
       <c r="G52" t="n">
-        <v>179.9</v>
+        <v>173.7</v>
       </c>
       <c r="H52" t="n">
-        <v>94.2</v>
+        <v>87.7</v>
       </c>
       <c r="I52" t="n">
         <v>16</v>
       </c>
       <c r="J52" t="n">
-        <v>-49.28</v>
+        <v>-51.72</v>
       </c>
       <c r="K52" t="n">
-        <v>209.19</v>
+        <v>215.77</v>
       </c>
       <c r="L52" t="n">
-        <v>214.92</v>
+        <v>221.89</v>
       </c>
     </row>
     <row r="53">
@@ -2266,25 +2266,25 @@
         <v>5.42</v>
       </c>
       <c r="F53" t="n">
-        <v>12.34</v>
+        <v>13.78</v>
       </c>
       <c r="G53" t="n">
-        <v>183.3</v>
+        <v>186.5</v>
       </c>
       <c r="H53" t="n">
-        <v>84.40000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="I53" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J53" t="n">
-        <v>199.97</v>
+        <v>234.97</v>
       </c>
       <c r="K53" t="n">
-        <v>37.17</v>
+        <v>-16.64</v>
       </c>
       <c r="L53" t="n">
-        <v>203.39</v>
+        <v>235.55</v>
       </c>
     </row>
     <row r="54">
@@ -2308,25 +2308,25 @@
         <v>5.53</v>
       </c>
       <c r="F54" t="n">
-        <v>11.91</v>
+        <v>14.14</v>
       </c>
       <c r="G54" t="n">
-        <v>198.7</v>
+        <v>177.9</v>
       </c>
       <c r="H54" t="n">
-        <v>94.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="I54" t="n">
         <v>17</v>
       </c>
       <c r="J54" t="n">
-        <v>249.82</v>
+        <v>275.87</v>
       </c>
       <c r="K54" t="n">
-        <v>-75.67</v>
+        <v>-120.75</v>
       </c>
       <c r="L54" t="n">
-        <v>261.03</v>
+        <v>301.14</v>
       </c>
     </row>
     <row r="55">
@@ -2350,25 +2350,25 @@
         <v>5.82</v>
       </c>
       <c r="F55" t="n">
-        <v>12.93</v>
+        <v>14.14</v>
       </c>
       <c r="G55" t="n">
-        <v>187.8</v>
+        <v>198.2</v>
       </c>
       <c r="H55" t="n">
-        <v>91.09999999999999</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="I55" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J55" t="n">
-        <v>-222.15</v>
+        <v>-236.84</v>
       </c>
       <c r="K55" t="n">
-        <v>-151.44</v>
+        <v>-184.08</v>
       </c>
       <c r="L55" t="n">
-        <v>268.86</v>
+        <v>299.97</v>
       </c>
     </row>
     <row r="56">
@@ -2392,25 +2392,25 @@
         <v>5.48</v>
       </c>
       <c r="F56" t="n">
-        <v>12.76</v>
+        <v>14.14</v>
       </c>
       <c r="G56" t="n">
-        <v>181.4</v>
+        <v>194.9</v>
       </c>
       <c r="H56" t="n">
-        <v>93.09999999999999</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="I56" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J56" t="n">
-        <v>-200.67</v>
+        <v>-224.6</v>
       </c>
       <c r="K56" t="n">
-        <v>-490.2</v>
+        <v>-523.5</v>
       </c>
       <c r="L56" t="n">
-        <v>529.6799999999999</v>
+        <v>569.65</v>
       </c>
     </row>
     <row r="57">
@@ -2434,25 +2434,25 @@
         <v>4.98</v>
       </c>
       <c r="F57" t="n">
-        <v>12.38</v>
+        <v>11.88</v>
       </c>
       <c r="G57" t="n">
-        <v>184.4</v>
+        <v>187.3</v>
       </c>
       <c r="H57" t="n">
-        <v>89.59999999999999</v>
+        <v>90</v>
       </c>
       <c r="I57" t="n">
         <v>16</v>
       </c>
       <c r="J57" t="n">
-        <v>262.51</v>
+        <v>306.12</v>
       </c>
       <c r="K57" t="n">
-        <v>159.56</v>
+        <v>124.08</v>
       </c>
       <c r="L57" t="n">
-        <v>307.2</v>
+        <v>330.31</v>
       </c>
     </row>
     <row r="58">
@@ -2476,25 +2476,25 @@
         <v>5.47</v>
       </c>
       <c r="F58" t="n">
-        <v>12.27</v>
+        <v>13.77</v>
       </c>
       <c r="G58" t="n">
-        <v>202</v>
+        <v>185</v>
       </c>
       <c r="H58" t="n">
-        <v>91.8</v>
+        <v>98.7</v>
       </c>
       <c r="I58" t="n">
         <v>17</v>
       </c>
       <c r="J58" t="n">
-        <v>-245.52</v>
+        <v>-241.47</v>
       </c>
       <c r="K58" t="n">
-        <v>-366.34</v>
+        <v>-438.21</v>
       </c>
       <c r="L58" t="n">
-        <v>441</v>
+        <v>500.33</v>
       </c>
     </row>
     <row r="59">
@@ -2518,25 +2518,25 @@
         <v>4.86</v>
       </c>
       <c r="F59" t="n">
-        <v>12.43</v>
+        <v>11.18</v>
       </c>
       <c r="G59" t="n">
-        <v>185.1</v>
+        <v>188.4</v>
       </c>
       <c r="H59" t="n">
-        <v>87</v>
+        <v>90.3</v>
       </c>
       <c r="I59" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J59" t="n">
-        <v>-53.58</v>
+        <v>-61.43</v>
       </c>
       <c r="K59" t="n">
-        <v>60.25</v>
+        <v>66.48</v>
       </c>
       <c r="L59" t="n">
-        <v>80.62</v>
+        <v>90.52</v>
       </c>
     </row>
     <row r="60">
@@ -2560,25 +2560,25 @@
         <v>6.56</v>
       </c>
       <c r="F60" t="n">
-        <v>11.72</v>
+        <v>14.14</v>
       </c>
       <c r="G60" t="n">
-        <v>187.2</v>
+        <v>174.1</v>
       </c>
       <c r="H60" t="n">
-        <v>92.8</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="I60" t="n">
         <v>16</v>
       </c>
       <c r="J60" t="n">
-        <v>26.41</v>
+        <v>29.29</v>
       </c>
       <c r="K60" t="n">
-        <v>-97.8</v>
+        <v>-106.42</v>
       </c>
       <c r="L60" t="n">
-        <v>101.3</v>
+        <v>110.37</v>
       </c>
     </row>
     <row r="61">
@@ -2602,25 +2602,25 @@
         <v>5.44</v>
       </c>
       <c r="F61" t="n">
-        <v>12.45</v>
+        <v>14.14</v>
       </c>
       <c r="G61" t="n">
-        <v>183.7</v>
+        <v>188.6</v>
       </c>
       <c r="H61" t="n">
-        <v>95.59999999999999</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="I61" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J61" t="n">
-        <v>-81.7</v>
+        <v>-88.39</v>
       </c>
       <c r="K61" t="n">
-        <v>-23.54</v>
+        <v>-27.5</v>
       </c>
       <c r="L61" t="n">
-        <v>85.02</v>
+        <v>92.56999999999999</v>
       </c>
     </row>
     <row r="62">
@@ -2644,25 +2644,25 @@
         <v>4.97</v>
       </c>
       <c r="F62" t="n">
-        <v>11.97</v>
+        <v>14.14</v>
       </c>
       <c r="G62" t="n">
-        <v>176.3</v>
+        <v>179</v>
       </c>
       <c r="H62" t="n">
-        <v>98.59999999999999</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="I62" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J62" t="n">
-        <v>104.5</v>
+        <v>114.41</v>
       </c>
       <c r="K62" t="n">
-        <v>-83.04000000000001</v>
+        <v>-95.5</v>
       </c>
       <c r="L62" t="n">
-        <v>133.47</v>
+        <v>149.03</v>
       </c>
     </row>
     <row r="63">
@@ -2686,25 +2686,25 @@
         <v>5.5</v>
       </c>
       <c r="F63" t="n">
-        <v>11.79</v>
+        <v>11.19</v>
       </c>
       <c r="G63" t="n">
-        <v>172.5</v>
+        <v>181.5</v>
       </c>
       <c r="H63" t="n">
         <v>88.90000000000001</v>
       </c>
       <c r="I63" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J63" t="n">
-        <v>-51.72</v>
+        <v>17.03</v>
       </c>
       <c r="K63" t="n">
-        <v>75.34</v>
+        <v>-136.78</v>
       </c>
       <c r="L63" t="n">
-        <v>91.38</v>
+        <v>137.84</v>
       </c>
     </row>
     <row r="64">
@@ -2725,28 +2725,28 @@
         <v>3</v>
       </c>
       <c r="E64" t="n">
-        <v>5.5</v>
+        <v>5.61</v>
       </c>
       <c r="F64" t="n">
-        <v>12.81</v>
+        <v>14.14</v>
       </c>
       <c r="G64" t="n">
-        <v>181.1</v>
+        <v>180.6</v>
       </c>
       <c r="H64" t="n">
-        <v>92.7</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="I64" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="J64" t="n">
-        <v>-71.95999999999999</v>
+        <v>98.92</v>
       </c>
       <c r="K64" t="n">
-        <v>53.41</v>
+        <v>40</v>
       </c>
       <c r="L64" t="n">
-        <v>89.61</v>
+        <v>106.7</v>
       </c>
     </row>
     <row r="65">
@@ -2767,28 +2767,28 @@
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>6.27</v>
+        <v>4.76</v>
       </c>
       <c r="F65" t="n">
-        <v>11.73</v>
+        <v>10.29</v>
       </c>
       <c r="G65" t="n">
-        <v>187.6</v>
+        <v>189.3</v>
       </c>
       <c r="H65" t="n">
-        <v>86.5</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="I65" t="n">
         <v>19</v>
       </c>
       <c r="J65" t="n">
-        <v>-109.8</v>
+        <v>-162.46</v>
       </c>
       <c r="K65" t="n">
-        <v>-190.61</v>
+        <v>51.88</v>
       </c>
       <c r="L65" t="n">
-        <v>219.97</v>
+        <v>170.54</v>
       </c>
     </row>
     <row r="66">
@@ -2809,28 +2809,28 @@
         <v>2</v>
       </c>
       <c r="E66" t="n">
-        <v>5.71</v>
+        <v>5.53</v>
       </c>
       <c r="F66" t="n">
-        <v>12.12</v>
+        <v>14.14</v>
       </c>
       <c r="G66" t="n">
-        <v>197.3</v>
+        <v>186</v>
       </c>
       <c r="H66" t="n">
-        <v>88.09999999999999</v>
+        <v>88.8</v>
       </c>
       <c r="I66" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J66" t="n">
-        <v>51.48</v>
+        <v>-162.01</v>
       </c>
       <c r="K66" t="n">
-        <v>-170.87</v>
+        <v>32.81</v>
       </c>
       <c r="L66" t="n">
-        <v>178.46</v>
+        <v>165.3</v>
       </c>
     </row>
     <row r="67">
@@ -2851,28 +2851,28 @@
         <v>3</v>
       </c>
       <c r="E67" t="n">
-        <v>5.62</v>
+        <v>5.23</v>
       </c>
       <c r="F67" t="n">
-        <v>11.33</v>
+        <v>14.14</v>
       </c>
       <c r="G67" t="n">
-        <v>177.4</v>
+        <v>198.6</v>
       </c>
       <c r="H67" t="n">
-        <v>96.09999999999999</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="I67" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J67" t="n">
-        <v>263.37</v>
+        <v>-56.2</v>
       </c>
       <c r="K67" t="n">
-        <v>-56.01</v>
+        <v>-248.06</v>
       </c>
       <c r="L67" t="n">
-        <v>269.26</v>
+        <v>254.34</v>
       </c>
     </row>
     <row r="68">
@@ -2893,28 +2893,28 @@
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>4.69</v>
+        <v>5.33</v>
       </c>
       <c r="F68" t="n">
-        <v>11.85</v>
+        <v>12.96</v>
       </c>
       <c r="G68" t="n">
-        <v>184.2</v>
+        <v>190.3</v>
       </c>
       <c r="H68" t="n">
-        <v>89.5</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I68" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J68" t="n">
-        <v>68.98999999999999</v>
+        <v>-297.31</v>
       </c>
       <c r="K68" t="n">
-        <v>-224.71</v>
+        <v>58.03</v>
       </c>
       <c r="L68" t="n">
-        <v>235.07</v>
+        <v>302.92</v>
       </c>
     </row>
     <row r="69">
@@ -2935,28 +2935,28 @@
         <v>2</v>
       </c>
       <c r="E69" t="n">
-        <v>5.74</v>
+        <v>6.27</v>
       </c>
       <c r="F69" t="n">
-        <v>12.55</v>
+        <v>14.14</v>
       </c>
       <c r="G69" t="n">
-        <v>184.6</v>
+        <v>171.9</v>
       </c>
       <c r="H69" t="n">
-        <v>89.3</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="I69" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J69" t="n">
-        <v>-206.1</v>
+        <v>-81.22</v>
       </c>
       <c r="K69" t="n">
-        <v>-310.8</v>
+        <v>352.93</v>
       </c>
       <c r="L69" t="n">
-        <v>372.93</v>
+        <v>362.15</v>
       </c>
     </row>
     <row r="70">
@@ -2977,28 +2977,28 @@
         <v>3</v>
       </c>
       <c r="E70" t="n">
-        <v>5.54</v>
+        <v>5.4</v>
       </c>
       <c r="F70" t="n">
-        <v>12.97</v>
+        <v>11.85</v>
       </c>
       <c r="G70" t="n">
-        <v>184.3</v>
+        <v>188.3</v>
       </c>
       <c r="H70" t="n">
-        <v>98</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="I70" t="n">
         <v>16</v>
       </c>
       <c r="J70" t="n">
-        <v>204.59</v>
+        <v>35</v>
       </c>
       <c r="K70" t="n">
-        <v>41.29</v>
+        <v>238.89</v>
       </c>
       <c r="L70" t="n">
-        <v>208.72</v>
+        <v>241.44</v>
       </c>
     </row>
     <row r="71">
@@ -3019,28 +3019,28 @@
         <v>1</v>
       </c>
       <c r="E71" t="n">
-        <v>5.15</v>
+        <v>5.37</v>
       </c>
       <c r="F71" t="n">
-        <v>12.29</v>
+        <v>13.37</v>
       </c>
       <c r="G71" t="n">
-        <v>172.2</v>
+        <v>185</v>
       </c>
       <c r="H71" t="n">
-        <v>89.3</v>
+        <v>89.2</v>
       </c>
       <c r="I71" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="J71" t="n">
-        <v>-184.79</v>
+        <v>-506.15</v>
       </c>
       <c r="K71" t="n">
-        <v>-197.29</v>
+        <v>25.63</v>
       </c>
       <c r="L71" t="n">
-        <v>270.32</v>
+        <v>506.8</v>
       </c>
     </row>
     <row r="72">
@@ -3061,28 +3061,28 @@
         <v>2</v>
       </c>
       <c r="E72" t="n">
-        <v>4.83</v>
+        <v>5.3</v>
       </c>
       <c r="F72" t="n">
-        <v>11.27</v>
+        <v>14.14</v>
       </c>
       <c r="G72" t="n">
-        <v>181.5</v>
+        <v>180</v>
       </c>
       <c r="H72" t="n">
-        <v>92.5</v>
+        <v>91.7</v>
       </c>
       <c r="I72" t="n">
         <v>16</v>
       </c>
       <c r="J72" t="n">
-        <v>88.03</v>
+        <v>397.62</v>
       </c>
       <c r="K72" t="n">
-        <v>-314.73</v>
+        <v>-24.1</v>
       </c>
       <c r="L72" t="n">
-        <v>326.8</v>
+        <v>398.35</v>
       </c>
     </row>
     <row r="73">
@@ -3103,28 +3103,28 @@
         <v>3</v>
       </c>
       <c r="E73" t="n">
-        <v>4.99</v>
+        <v>6.45</v>
       </c>
       <c r="F73" t="n">
-        <v>12.46</v>
+        <v>14.14</v>
       </c>
       <c r="G73" t="n">
-        <v>189.1</v>
+        <v>190.7</v>
       </c>
       <c r="H73" t="n">
-        <v>100</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="I73" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J73" t="n">
-        <v>295.87</v>
+        <v>-302.77</v>
       </c>
       <c r="K73" t="n">
-        <v>145.49</v>
+        <v>-421.14</v>
       </c>
       <c r="L73" t="n">
-        <v>329.71</v>
+        <v>518.6799999999999</v>
       </c>
     </row>
     <row r="74">
@@ -3145,28 +3145,28 @@
         <v>1</v>
       </c>
       <c r="E74" t="n">
-        <v>6.05</v>
+        <v>5.36</v>
       </c>
       <c r="F74" t="n">
-        <v>12.62</v>
+        <v>14.14</v>
       </c>
       <c r="G74" t="n">
-        <v>181.9</v>
+        <v>182.3</v>
       </c>
       <c r="H74" t="n">
-        <v>88.90000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="I74" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J74" t="n">
-        <v>-50.95</v>
+        <v>-22.88</v>
       </c>
       <c r="K74" t="n">
-        <v>-51.96</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="L74" t="n">
-        <v>72.77</v>
+        <v>84.48</v>
       </c>
     </row>
     <row r="75">
@@ -3187,28 +3187,28 @@
         <v>2</v>
       </c>
       <c r="E75" t="n">
-        <v>5.68</v>
+        <v>4.67</v>
       </c>
       <c r="F75" t="n">
-        <v>11.99</v>
+        <v>10.62</v>
       </c>
       <c r="G75" t="n">
-        <v>179.1</v>
+        <v>178.4</v>
       </c>
       <c r="H75" t="n">
-        <v>81.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="I75" t="n">
         <v>16</v>
       </c>
       <c r="J75" t="n">
-        <v>-64.26000000000001</v>
+        <v>85.19</v>
       </c>
       <c r="K75" t="n">
-        <v>-63.87</v>
+        <v>-23.32</v>
       </c>
       <c r="L75" t="n">
-        <v>90.59999999999999</v>
+        <v>88.31999999999999</v>
       </c>
     </row>
     <row r="76">
@@ -3229,28 +3229,28 @@
         <v>3</v>
       </c>
       <c r="E76" t="n">
-        <v>5.49</v>
+        <v>5.16</v>
       </c>
       <c r="F76" t="n">
-        <v>12.28</v>
+        <v>14.14</v>
       </c>
       <c r="G76" t="n">
-        <v>177.5</v>
+        <v>178.4</v>
       </c>
       <c r="H76" t="n">
-        <v>89.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="I76" t="n">
         <v>16</v>
       </c>
       <c r="J76" t="n">
-        <v>-65.08</v>
+        <v>-27.87</v>
       </c>
       <c r="K76" t="n">
-        <v>-63.54</v>
+        <v>73.73999999999999</v>
       </c>
       <c r="L76" t="n">
-        <v>90.95</v>
+        <v>78.83</v>
       </c>
     </row>
     <row r="77">
@@ -3271,28 +3271,28 @@
         <v>1</v>
       </c>
       <c r="E77" t="n">
-        <v>5.81</v>
+        <v>5.58</v>
       </c>
       <c r="F77" t="n">
-        <v>11.89</v>
+        <v>12.6</v>
       </c>
       <c r="G77" t="n">
-        <v>191.3</v>
+        <v>176</v>
       </c>
       <c r="H77" t="n">
-        <v>90.5</v>
+        <v>89.8</v>
       </c>
       <c r="I77" t="n">
         <v>16</v>
       </c>
       <c r="J77" t="n">
-        <v>-22.28</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="K77" t="n">
-        <v>-127.49</v>
+        <v>-59.61</v>
       </c>
       <c r="L77" t="n">
-        <v>129.43</v>
+        <v>103.49</v>
       </c>
     </row>
     <row r="78">
@@ -3313,28 +3313,28 @@
         <v>2</v>
       </c>
       <c r="E78" t="n">
-        <v>4.98</v>
+        <v>5.19</v>
       </c>
       <c r="F78" t="n">
-        <v>12.26</v>
+        <v>14.14</v>
       </c>
       <c r="G78" t="n">
-        <v>177.5</v>
+        <v>173.7</v>
       </c>
       <c r="H78" t="n">
-        <v>89.2</v>
+        <v>81.5</v>
       </c>
       <c r="I78" t="n">
         <v>16</v>
       </c>
       <c r="J78" t="n">
-        <v>-129.41</v>
+        <v>124.63</v>
       </c>
       <c r="K78" t="n">
-        <v>-88.5</v>
+        <v>12.98</v>
       </c>
       <c r="L78" t="n">
-        <v>156.77</v>
+        <v>125.3</v>
       </c>
     </row>
     <row r="79">
@@ -3355,28 +3355,28 @@
         <v>3</v>
       </c>
       <c r="E79" t="n">
-        <v>5.24</v>
+        <v>5.9</v>
       </c>
       <c r="F79" t="n">
-        <v>11.85</v>
+        <v>13.31</v>
       </c>
       <c r="G79" t="n">
-        <v>176.6</v>
+        <v>190.1</v>
       </c>
       <c r="H79" t="n">
-        <v>93.7</v>
+        <v>90.8</v>
       </c>
       <c r="I79" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J79" t="n">
-        <v>9.73</v>
+        <v>73.26000000000001</v>
       </c>
       <c r="K79" t="n">
-        <v>75.90000000000001</v>
+        <v>3.76</v>
       </c>
       <c r="L79" t="n">
-        <v>76.53</v>
+        <v>73.36</v>
       </c>
     </row>
     <row r="80">
@@ -3397,28 +3397,28 @@
         <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>5.55</v>
+        <v>6.3</v>
       </c>
       <c r="F80" t="n">
-        <v>12.62</v>
+        <v>12.75</v>
       </c>
       <c r="G80" t="n">
-        <v>191.9</v>
+        <v>195.2</v>
       </c>
       <c r="H80" t="n">
-        <v>91.2</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="I80" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J80" t="n">
-        <v>-238.13</v>
+        <v>-254.6</v>
       </c>
       <c r="K80" t="n">
-        <v>90.84999999999999</v>
+        <v>-35.71</v>
       </c>
       <c r="L80" t="n">
-        <v>254.88</v>
+        <v>257.09</v>
       </c>
     </row>
     <row r="81">
@@ -3439,28 +3439,28 @@
         <v>2</v>
       </c>
       <c r="E81" t="n">
-        <v>6.09</v>
+        <v>5.99</v>
       </c>
       <c r="F81" t="n">
-        <v>13.02</v>
+        <v>14.14</v>
       </c>
       <c r="G81" t="n">
-        <v>193.1</v>
+        <v>185.8</v>
       </c>
       <c r="H81" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="I81" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J81" t="n">
-        <v>-67.41</v>
+        <v>-128.76</v>
       </c>
       <c r="K81" t="n">
-        <v>-172.67</v>
+        <v>205.81</v>
       </c>
       <c r="L81" t="n">
-        <v>185.36</v>
+        <v>242.77</v>
       </c>
     </row>
     <row r="82">
@@ -3481,28 +3481,28 @@
         <v>3</v>
       </c>
       <c r="E82" t="n">
-        <v>5.63</v>
+        <v>6.33</v>
       </c>
       <c r="F82" t="n">
-        <v>13.01</v>
+        <v>14.14</v>
       </c>
       <c r="G82" t="n">
-        <v>202.1</v>
+        <v>190.8</v>
       </c>
       <c r="H82" t="n">
-        <v>86.5</v>
+        <v>94</v>
       </c>
       <c r="I82" t="n">
         <v>18</v>
       </c>
       <c r="J82" t="n">
-        <v>-140.23</v>
+        <v>204.99</v>
       </c>
       <c r="K82" t="n">
-        <v>104.72</v>
+        <v>44.03</v>
       </c>
       <c r="L82" t="n">
-        <v>175.02</v>
+        <v>209.66</v>
       </c>
     </row>
     <row r="83">
@@ -3523,28 +3523,28 @@
         <v>1</v>
       </c>
       <c r="E83" t="n">
-        <v>5.9</v>
+        <v>5.94</v>
       </c>
       <c r="F83" t="n">
-        <v>12.55</v>
+        <v>14.14</v>
       </c>
       <c r="G83" t="n">
-        <v>191.6</v>
+        <v>181.3</v>
       </c>
       <c r="H83" t="n">
-        <v>93.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="I83" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J83" t="n">
-        <v>-341.47</v>
+        <v>299.11</v>
       </c>
       <c r="K83" t="n">
-        <v>-24.25</v>
+        <v>237.66</v>
       </c>
       <c r="L83" t="n">
-        <v>342.33</v>
+        <v>382.03</v>
       </c>
     </row>
     <row r="84">
@@ -3565,28 +3565,28 @@
         <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>5.44</v>
+        <v>6.19</v>
       </c>
       <c r="F84" t="n">
-        <v>12.84</v>
+        <v>14.14</v>
       </c>
       <c r="G84" t="n">
-        <v>199.5</v>
+        <v>187.3</v>
       </c>
       <c r="H84" t="n">
-        <v>97.3</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="I84" t="n">
         <v>16</v>
       </c>
       <c r="J84" t="n">
-        <v>260.18</v>
+        <v>181.85</v>
       </c>
       <c r="K84" t="n">
-        <v>-35.94</v>
+        <v>-176.71</v>
       </c>
       <c r="L84" t="n">
-        <v>262.65</v>
+        <v>253.57</v>
       </c>
     </row>
     <row r="85">
@@ -3607,28 +3607,28 @@
         <v>3</v>
       </c>
       <c r="E85" t="n">
-        <v>5.74</v>
+        <v>5.46</v>
       </c>
       <c r="F85" t="n">
-        <v>12.28</v>
+        <v>14.14</v>
       </c>
       <c r="G85" t="n">
-        <v>175.3</v>
+        <v>187.7</v>
       </c>
       <c r="H85" t="n">
-        <v>90.8</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="I85" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J85" t="n">
-        <v>317.32</v>
+        <v>-51.56</v>
       </c>
       <c r="K85" t="n">
-        <v>119.41</v>
+        <v>-297.24</v>
       </c>
       <c r="L85" t="n">
-        <v>339.04</v>
+        <v>301.68</v>
       </c>
     </row>
     <row r="86">
@@ -3649,28 +3649,28 @@
         <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>5.68</v>
+        <v>5.62</v>
       </c>
       <c r="F86" t="n">
-        <v>11.87</v>
+        <v>12.55</v>
       </c>
       <c r="G86" t="n">
-        <v>184.1</v>
+        <v>188.8</v>
       </c>
       <c r="H86" t="n">
-        <v>90.8</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="I86" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J86" t="n">
-        <v>-228.41</v>
+        <v>-109.47</v>
       </c>
       <c r="K86" t="n">
-        <v>-448.38</v>
+        <v>357.46</v>
       </c>
       <c r="L86" t="n">
-        <v>503.2</v>
+        <v>373.85</v>
       </c>
     </row>
     <row r="87">
@@ -3691,28 +3691,28 @@
         <v>2</v>
       </c>
       <c r="E87" t="n">
-        <v>5.88</v>
+        <v>6.1</v>
       </c>
       <c r="F87" t="n">
-        <v>12.72</v>
+        <v>14.14</v>
       </c>
       <c r="G87" t="n">
-        <v>193.7</v>
+        <v>188.5</v>
       </c>
       <c r="H87" t="n">
-        <v>90.09999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="I87" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J87" t="n">
-        <v>-7.69</v>
+        <v>464.78</v>
       </c>
       <c r="K87" t="n">
-        <v>-412.22</v>
+        <v>266.55</v>
       </c>
       <c r="L87" t="n">
-        <v>412.29</v>
+        <v>535.79</v>
       </c>
     </row>
     <row r="88">
@@ -3733,28 +3733,28 @@
         <v>3</v>
       </c>
       <c r="E88" t="n">
-        <v>5.26</v>
+        <v>5.63</v>
       </c>
       <c r="F88" t="n">
-        <v>12.74</v>
+        <v>13.92</v>
       </c>
       <c r="G88" t="n">
-        <v>196</v>
+        <v>184.1</v>
       </c>
       <c r="H88" t="n">
-        <v>92.09999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="I88" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J88" t="n">
-        <v>-373.51</v>
+        <v>102.32</v>
       </c>
       <c r="K88" t="n">
-        <v>-159.12</v>
+        <v>-411.91</v>
       </c>
       <c r="L88" t="n">
-        <v>405.99</v>
+        <v>424.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
after markdown and merged model fix
</commit_message>
<xml_diff>
--- a/output/2024-04-01.xlsx
+++ b/output/2024-04-01.xlsx
@@ -640,13 +640,13 @@
         <v>16</v>
       </c>
       <c r="J14" t="n">
-        <v>-29.03</v>
+        <v>-32.73</v>
       </c>
       <c r="K14" t="n">
-        <v>-64.43000000000001</v>
+        <v>-72.65000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>70.66</v>
+        <v>79.68000000000001</v>
       </c>
     </row>
     <row r="15">
@@ -682,13 +682,13 @@
         <v>16</v>
       </c>
       <c r="J15" t="n">
-        <v>-37.36</v>
+        <v>-42.13</v>
       </c>
       <c r="K15" t="n">
-        <v>60.78</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="L15" t="n">
-        <v>71.34</v>
+        <v>80.45</v>
       </c>
     </row>
     <row r="16">
@@ -724,13 +724,13 @@
         <v>16</v>
       </c>
       <c r="J16" t="n">
-        <v>-82.02</v>
+        <v>-92.5</v>
       </c>
       <c r="K16" t="n">
-        <v>-63.26</v>
+        <v>-71.34</v>
       </c>
       <c r="L16" t="n">
-        <v>103.59</v>
+        <v>116.82</v>
       </c>
     </row>
     <row r="17">
@@ -766,13 +766,13 @@
         <v>18</v>
       </c>
       <c r="J17" t="n">
-        <v>41.86</v>
+        <v>46.06</v>
       </c>
       <c r="K17" t="n">
-        <v>96.31</v>
+        <v>105.99</v>
       </c>
       <c r="L17" t="n">
-        <v>105.02</v>
+        <v>115.57</v>
       </c>
     </row>
     <row r="18">
@@ -808,13 +808,13 @@
         <v>16</v>
       </c>
       <c r="J18" t="n">
-        <v>15.27</v>
+        <v>17.26</v>
       </c>
       <c r="K18" t="n">
-        <v>22.72</v>
+        <v>25.69</v>
       </c>
       <c r="L18" t="n">
-        <v>27.38</v>
+        <v>30.95</v>
       </c>
     </row>
     <row r="19">
@@ -850,13 +850,13 @@
         <v>18</v>
       </c>
       <c r="J19" t="n">
-        <v>98.97</v>
+        <v>106.47</v>
       </c>
       <c r="K19" t="n">
-        <v>-71.65000000000001</v>
+        <v>-77.09</v>
       </c>
       <c r="L19" t="n">
-        <v>122.18</v>
+        <v>131.45</v>
       </c>
     </row>
     <row r="20">
@@ -892,13 +892,13 @@
         <v>18</v>
       </c>
       <c r="J20" t="n">
-        <v>150.09</v>
+        <v>165.85</v>
       </c>
       <c r="K20" t="n">
-        <v>-49.63</v>
+        <v>-54.84</v>
       </c>
       <c r="L20" t="n">
-        <v>158.08</v>
+        <v>174.68</v>
       </c>
     </row>
     <row r="21">
@@ -934,13 +934,13 @@
         <v>16</v>
       </c>
       <c r="J21" t="n">
-        <v>-159.42</v>
+        <v>-181.17</v>
       </c>
       <c r="K21" t="n">
-        <v>-76.23999999999999</v>
+        <v>-86.64</v>
       </c>
       <c r="L21" t="n">
-        <v>176.72</v>
+        <v>200.82</v>
       </c>
     </row>
     <row r="22">
@@ -976,13 +976,13 @@
         <v>16</v>
       </c>
       <c r="J22" t="n">
-        <v>-101.13</v>
+        <v>-114.74</v>
       </c>
       <c r="K22" t="n">
-        <v>-98.84</v>
+        <v>-112.14</v>
       </c>
       <c r="L22" t="n">
-        <v>141.41</v>
+        <v>160.43</v>
       </c>
     </row>
     <row r="23">
@@ -1018,13 +1018,13 @@
         <v>18</v>
       </c>
       <c r="J23" t="n">
-        <v>99.72</v>
+        <v>111.25</v>
       </c>
       <c r="K23" t="n">
-        <v>-130.44</v>
+        <v>-145.52</v>
       </c>
       <c r="L23" t="n">
-        <v>164.19</v>
+        <v>183.18</v>
       </c>
     </row>
     <row r="24">
@@ -1060,13 +1060,13 @@
         <v>16</v>
       </c>
       <c r="J24" t="n">
-        <v>47.06</v>
+        <v>54.01</v>
       </c>
       <c r="K24" t="n">
-        <v>-228.42</v>
+        <v>-262.12</v>
       </c>
       <c r="L24" t="n">
-        <v>233.21</v>
+        <v>267.62</v>
       </c>
     </row>
     <row r="25">
@@ -1102,13 +1102,13 @@
         <v>16</v>
       </c>
       <c r="J25" t="n">
-        <v>-187.78</v>
+        <v>-213.95</v>
       </c>
       <c r="K25" t="n">
-        <v>-134.63</v>
+        <v>-153.39</v>
       </c>
       <c r="L25" t="n">
-        <v>231.05</v>
+        <v>263.26</v>
       </c>
     </row>
     <row r="26">
@@ -1144,13 +1144,13 @@
         <v>19</v>
       </c>
       <c r="J26" t="n">
-        <v>263.38</v>
+        <v>292.48</v>
       </c>
       <c r="K26" t="n">
-        <v>-540.3200000000001</v>
+        <v>-600.03</v>
       </c>
       <c r="L26" t="n">
-        <v>601.1</v>
+        <v>667.52</v>
       </c>
     </row>
     <row r="27">
@@ -1186,13 +1186,13 @@
         <v>16</v>
       </c>
       <c r="J27" t="n">
-        <v>-405.39</v>
+        <v>-469.03</v>
       </c>
       <c r="K27" t="n">
-        <v>119.21</v>
+        <v>137.92</v>
       </c>
       <c r="L27" t="n">
-        <v>422.56</v>
+        <v>488.89</v>
       </c>
     </row>
     <row r="28">
@@ -1228,13 +1228,13 @@
         <v>16</v>
       </c>
       <c r="J28" t="n">
-        <v>378.9</v>
+        <v>438.3</v>
       </c>
       <c r="K28" t="n">
-        <v>185.34</v>
+        <v>214.39</v>
       </c>
       <c r="L28" t="n">
-        <v>421.81</v>
+        <v>487.92</v>
       </c>
     </row>
     <row r="29">
@@ -1270,13 +1270,13 @@
         <v>16</v>
       </c>
       <c r="J29" t="n">
-        <v>63.85</v>
+        <v>72.05</v>
       </c>
       <c r="K29" t="n">
-        <v>-80.78</v>
+        <v>-91.16</v>
       </c>
       <c r="L29" t="n">
-        <v>102.97</v>
+        <v>116.19</v>
       </c>
     </row>
     <row r="30">
@@ -1312,13 +1312,13 @@
         <v>18</v>
       </c>
       <c r="J30" t="n">
-        <v>42.26</v>
+        <v>46.37</v>
       </c>
       <c r="K30" t="n">
-        <v>-96.51000000000001</v>
+        <v>-105.89</v>
       </c>
       <c r="L30" t="n">
-        <v>105.36</v>
+        <v>115.6</v>
       </c>
     </row>
     <row r="31">
@@ -1354,13 +1354,13 @@
         <v>16</v>
       </c>
       <c r="J31" t="n">
-        <v>2.35</v>
+        <v>2.65</v>
       </c>
       <c r="K31" t="n">
-        <v>-91.91</v>
+        <v>-103.79</v>
       </c>
       <c r="L31" t="n">
-        <v>91.94</v>
+        <v>103.82</v>
       </c>
     </row>
     <row r="32">
@@ -1396,13 +1396,13 @@
         <v>17</v>
       </c>
       <c r="J32" t="n">
-        <v>75.55</v>
+        <v>84.28</v>
       </c>
       <c r="K32" t="n">
-        <v>-11.4</v>
+        <v>-12.72</v>
       </c>
       <c r="L32" t="n">
-        <v>76.41</v>
+        <v>85.23</v>
       </c>
     </row>
     <row r="33">
@@ -1438,13 +1438,13 @@
         <v>16</v>
       </c>
       <c r="J33" t="n">
-        <v>44.15</v>
+        <v>49.82</v>
       </c>
       <c r="K33" t="n">
-        <v>82.78</v>
+        <v>93.41</v>
       </c>
       <c r="L33" t="n">
-        <v>93.81999999999999</v>
+        <v>105.87</v>
       </c>
     </row>
     <row r="34">
@@ -1480,13 +1480,13 @@
         <v>19</v>
       </c>
       <c r="J34" t="n">
-        <v>-93.38</v>
+        <v>-101.18</v>
       </c>
       <c r="K34" t="n">
-        <v>-28.12</v>
+        <v>-30.47</v>
       </c>
       <c r="L34" t="n">
-        <v>97.52</v>
+        <v>105.67</v>
       </c>
     </row>
     <row r="35">
@@ -1522,13 +1522,13 @@
         <v>16</v>
       </c>
       <c r="J35" t="n">
-        <v>-163.23</v>
+        <v>-185.14</v>
       </c>
       <c r="K35" t="n">
-        <v>-15.31</v>
+        <v>-17.37</v>
       </c>
       <c r="L35" t="n">
-        <v>163.95</v>
+        <v>185.95</v>
       </c>
     </row>
     <row r="36">
@@ -1564,13 +1564,13 @@
         <v>16</v>
       </c>
       <c r="J36" t="n">
-        <v>251.35</v>
+        <v>284.92</v>
       </c>
       <c r="K36" t="n">
-        <v>-58.45</v>
+        <v>-66.25</v>
       </c>
       <c r="L36" t="n">
-        <v>258.05</v>
+        <v>292.53</v>
       </c>
     </row>
     <row r="37">
@@ -1606,13 +1606,13 @@
         <v>16</v>
       </c>
       <c r="J37" t="n">
-        <v>-157.58</v>
+        <v>-179.03</v>
       </c>
       <c r="K37" t="n">
-        <v>-105.56</v>
+        <v>-119.93</v>
       </c>
       <c r="L37" t="n">
-        <v>189.67</v>
+        <v>215.49</v>
       </c>
     </row>
     <row r="38">
@@ -1648,13 +1648,13 @@
         <v>16</v>
       </c>
       <c r="J38" t="n">
-        <v>-190.82</v>
+        <v>-219.22</v>
       </c>
       <c r="K38" t="n">
-        <v>34.52</v>
+        <v>39.66</v>
       </c>
       <c r="L38" t="n">
-        <v>193.91</v>
+        <v>222.78</v>
       </c>
     </row>
     <row r="39">
@@ -1690,13 +1690,13 @@
         <v>16</v>
       </c>
       <c r="J39" t="n">
-        <v>-191.72</v>
+        <v>-220.32</v>
       </c>
       <c r="K39" t="n">
-        <v>-145.95</v>
+        <v>-167.72</v>
       </c>
       <c r="L39" t="n">
-        <v>240.95</v>
+        <v>276.89</v>
       </c>
     </row>
     <row r="40">
@@ -1732,13 +1732,13 @@
         <v>17</v>
       </c>
       <c r="J40" t="n">
-        <v>122.2</v>
+        <v>138.5</v>
       </c>
       <c r="K40" t="n">
-        <v>-363.42</v>
+        <v>-411.88</v>
       </c>
       <c r="L40" t="n">
-        <v>383.42</v>
+        <v>434.54</v>
       </c>
     </row>
     <row r="41">
@@ -1774,13 +1774,13 @@
         <v>16</v>
       </c>
       <c r="J41" t="n">
-        <v>260.71</v>
+        <v>301.26</v>
       </c>
       <c r="K41" t="n">
-        <v>227.17</v>
+        <v>262.5</v>
       </c>
       <c r="L41" t="n">
-        <v>345.8</v>
+        <v>399.58</v>
       </c>
     </row>
     <row r="42">
@@ -1816,13 +1816,13 @@
         <v>16</v>
       </c>
       <c r="J42" t="n">
-        <v>-159.67</v>
+        <v>-185.09</v>
       </c>
       <c r="K42" t="n">
-        <v>-469.29</v>
+        <v>-543.99</v>
       </c>
       <c r="L42" t="n">
-        <v>495.71</v>
+        <v>574.61</v>
       </c>
     </row>
     <row r="43">
@@ -1858,13 +1858,13 @@
         <v>16</v>
       </c>
       <c r="J43" t="n">
-        <v>192.62</v>
+        <v>222.85</v>
       </c>
       <c r="K43" t="n">
-        <v>-245.2</v>
+        <v>-283.68</v>
       </c>
       <c r="L43" t="n">
-        <v>311.81</v>
+        <v>360.74</v>
       </c>
     </row>
     <row r="44">
@@ -1900,13 +1900,13 @@
         <v>19</v>
       </c>
       <c r="J44" t="n">
-        <v>56.24</v>
+        <v>61.01</v>
       </c>
       <c r="K44" t="n">
-        <v>-32.12</v>
+        <v>-34.85</v>
       </c>
       <c r="L44" t="n">
-        <v>64.77</v>
+        <v>70.26000000000001</v>
       </c>
     </row>
     <row r="45">
@@ -1942,13 +1942,13 @@
         <v>16</v>
       </c>
       <c r="J45" t="n">
-        <v>88.28</v>
+        <v>99.53</v>
       </c>
       <c r="K45" t="n">
-        <v>25.53</v>
+        <v>28.78</v>
       </c>
       <c r="L45" t="n">
-        <v>91.90000000000001</v>
+        <v>103.61</v>
       </c>
     </row>
     <row r="46">
@@ -1984,13 +1984,13 @@
         <v>16</v>
       </c>
       <c r="J46" t="n">
-        <v>77.02</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="K46" t="n">
-        <v>-65.62</v>
+        <v>-74.04000000000001</v>
       </c>
       <c r="L46" t="n">
-        <v>101.18</v>
+        <v>114.16</v>
       </c>
     </row>
     <row r="47">
@@ -2026,13 +2026,13 @@
         <v>16</v>
       </c>
       <c r="J47" t="n">
-        <v>-66.08</v>
+        <v>-74.5</v>
       </c>
       <c r="K47" t="n">
-        <v>-64.54000000000001</v>
+        <v>-72.77</v>
       </c>
       <c r="L47" t="n">
-        <v>92.37</v>
+        <v>104.15</v>
       </c>
     </row>
     <row r="48">
@@ -2068,13 +2068,13 @@
         <v>16</v>
       </c>
       <c r="J48" t="n">
-        <v>33.83</v>
+        <v>37.34</v>
       </c>
       <c r="K48" t="n">
-        <v>88.88</v>
+        <v>98.11</v>
       </c>
       <c r="L48" t="n">
-        <v>95.09999999999999</v>
+        <v>104.97</v>
       </c>
     </row>
     <row r="49">
@@ -2110,13 +2110,13 @@
         <v>16</v>
       </c>
       <c r="J49" t="n">
-        <v>13.76</v>
+        <v>15.53</v>
       </c>
       <c r="K49" t="n">
-        <v>83.54000000000001</v>
+        <v>94.29000000000001</v>
       </c>
       <c r="L49" t="n">
-        <v>84.66</v>
+        <v>95.56</v>
       </c>
     </row>
     <row r="50">
@@ -2152,13 +2152,13 @@
         <v>17</v>
       </c>
       <c r="J50" t="n">
-        <v>130.92</v>
+        <v>146.46</v>
       </c>
       <c r="K50" t="n">
-        <v>73.15000000000001</v>
+        <v>81.83</v>
       </c>
       <c r="L50" t="n">
-        <v>149.97</v>
+        <v>167.77</v>
       </c>
     </row>
     <row r="51">
@@ -2194,13 +2194,13 @@
         <v>16</v>
       </c>
       <c r="J51" t="n">
-        <v>-45.93</v>
+        <v>-52.05</v>
       </c>
       <c r="K51" t="n">
-        <v>-257.81</v>
+        <v>-292.14</v>
       </c>
       <c r="L51" t="n">
-        <v>261.87</v>
+        <v>296.74</v>
       </c>
     </row>
     <row r="52">
@@ -2236,13 +2236,13 @@
         <v>16</v>
       </c>
       <c r="J52" t="n">
-        <v>-51.72</v>
+        <v>-58.73</v>
       </c>
       <c r="K52" t="n">
-        <v>215.77</v>
+        <v>245</v>
       </c>
       <c r="L52" t="n">
-        <v>221.89</v>
+        <v>251.94</v>
       </c>
     </row>
     <row r="53">
@@ -2278,13 +2278,13 @@
         <v>16</v>
       </c>
       <c r="J53" t="n">
-        <v>234.97</v>
+        <v>270.1</v>
       </c>
       <c r="K53" t="n">
-        <v>-16.64</v>
+        <v>-19.12</v>
       </c>
       <c r="L53" t="n">
-        <v>235.55</v>
+        <v>270.78</v>
       </c>
     </row>
     <row r="54">
@@ -2320,13 +2320,13 @@
         <v>17</v>
       </c>
       <c r="J54" t="n">
-        <v>275.87</v>
+        <v>312.99</v>
       </c>
       <c r="K54" t="n">
-        <v>-120.75</v>
+        <v>-136.99</v>
       </c>
       <c r="L54" t="n">
-        <v>301.14</v>
+        <v>341.66</v>
       </c>
     </row>
     <row r="55">
@@ -2362,13 +2362,13 @@
         <v>18</v>
       </c>
       <c r="J55" t="n">
-        <v>-236.84</v>
+        <v>-265.12</v>
       </c>
       <c r="K55" t="n">
-        <v>-184.08</v>
+        <v>-206.06</v>
       </c>
       <c r="L55" t="n">
-        <v>299.97</v>
+        <v>335.78</v>
       </c>
     </row>
     <row r="56">
@@ -2404,13 +2404,13 @@
         <v>18</v>
       </c>
       <c r="J56" t="n">
-        <v>-224.6</v>
+        <v>-253.86</v>
       </c>
       <c r="K56" t="n">
-        <v>-523.5</v>
+        <v>-591.7</v>
       </c>
       <c r="L56" t="n">
-        <v>569.65</v>
+        <v>643.86</v>
       </c>
     </row>
     <row r="57">
@@ -2446,13 +2446,13 @@
         <v>16</v>
       </c>
       <c r="J57" t="n">
-        <v>306.12</v>
+        <v>354.7</v>
       </c>
       <c r="K57" t="n">
-        <v>124.08</v>
+        <v>143.77</v>
       </c>
       <c r="L57" t="n">
-        <v>330.31</v>
+        <v>382.73</v>
       </c>
     </row>
     <row r="58">
@@ -2488,13 +2488,13 @@
         <v>17</v>
       </c>
       <c r="J58" t="n">
-        <v>-241.47</v>
+        <v>-276.77</v>
       </c>
       <c r="K58" t="n">
-        <v>-438.21</v>
+        <v>-502.28</v>
       </c>
       <c r="L58" t="n">
-        <v>500.33</v>
+        <v>573.48</v>
       </c>
     </row>
     <row r="59">
@@ -2530,13 +2530,13 @@
         <v>16</v>
       </c>
       <c r="J59" t="n">
-        <v>-61.43</v>
+        <v>-69.38</v>
       </c>
       <c r="K59" t="n">
-        <v>66.48</v>
+        <v>75.08</v>
       </c>
       <c r="L59" t="n">
-        <v>90.52</v>
+        <v>102.23</v>
       </c>
     </row>
     <row r="60">
@@ -2572,13 +2572,13 @@
         <v>16</v>
       </c>
       <c r="J60" t="n">
-        <v>29.29</v>
+        <v>31.73</v>
       </c>
       <c r="K60" t="n">
-        <v>-106.42</v>
+        <v>-115.28</v>
       </c>
       <c r="L60" t="n">
-        <v>110.37</v>
+        <v>119.56</v>
       </c>
     </row>
     <row r="61">
@@ -2614,13 +2614,13 @@
         <v>19</v>
       </c>
       <c r="J61" t="n">
-        <v>-88.39</v>
+        <v>-95.47</v>
       </c>
       <c r="K61" t="n">
-        <v>-27.5</v>
+        <v>-29.7</v>
       </c>
       <c r="L61" t="n">
-        <v>92.56999999999999</v>
+        <v>99.98</v>
       </c>
     </row>
     <row r="62">
@@ -2656,13 +2656,13 @@
         <v>16</v>
       </c>
       <c r="J62" t="n">
-        <v>114.41</v>
+        <v>129.18</v>
       </c>
       <c r="K62" t="n">
-        <v>-95.5</v>
+        <v>-107.82</v>
       </c>
       <c r="L62" t="n">
-        <v>149.03</v>
+        <v>168.26</v>
       </c>
     </row>
     <row r="63">
@@ -2698,13 +2698,13 @@
         <v>16</v>
       </c>
       <c r="J63" t="n">
-        <v>17.03</v>
+        <v>19.18</v>
       </c>
       <c r="K63" t="n">
-        <v>-136.78</v>
+        <v>-154.12</v>
       </c>
       <c r="L63" t="n">
-        <v>137.84</v>
+        <v>155.3</v>
       </c>
     </row>
     <row r="64">
@@ -2740,13 +2740,13 @@
         <v>16</v>
       </c>
       <c r="J64" t="n">
-        <v>98.92</v>
+        <v>110.21</v>
       </c>
       <c r="K64" t="n">
-        <v>40</v>
+        <v>44.56</v>
       </c>
       <c r="L64" t="n">
-        <v>106.7</v>
+        <v>118.88</v>
       </c>
     </row>
     <row r="65">
@@ -2782,13 +2782,13 @@
         <v>19</v>
       </c>
       <c r="J65" t="n">
-        <v>-162.46</v>
+        <v>-176.82</v>
       </c>
       <c r="K65" t="n">
-        <v>51.88</v>
+        <v>56.47</v>
       </c>
       <c r="L65" t="n">
-        <v>170.54</v>
+        <v>185.62</v>
       </c>
     </row>
     <row r="66">
@@ -2824,13 +2824,13 @@
         <v>17</v>
       </c>
       <c r="J66" t="n">
-        <v>-162.01</v>
+        <v>-181.17</v>
       </c>
       <c r="K66" t="n">
-        <v>32.81</v>
+        <v>36.69</v>
       </c>
       <c r="L66" t="n">
-        <v>165.3</v>
+        <v>184.85</v>
       </c>
     </row>
     <row r="67">
@@ -2866,13 +2866,13 @@
         <v>16</v>
       </c>
       <c r="J67" t="n">
-        <v>-56.2</v>
+        <v>-63.72</v>
       </c>
       <c r="K67" t="n">
-        <v>-248.06</v>
+        <v>-281.23</v>
       </c>
       <c r="L67" t="n">
-        <v>254.34</v>
+        <v>288.36</v>
       </c>
     </row>
     <row r="68">
@@ -2908,13 +2908,13 @@
         <v>16</v>
       </c>
       <c r="J68" t="n">
-        <v>-297.31</v>
+        <v>-341.69</v>
       </c>
       <c r="K68" t="n">
-        <v>58.03</v>
+        <v>66.69</v>
       </c>
       <c r="L68" t="n">
-        <v>302.92</v>
+        <v>348.14</v>
       </c>
     </row>
     <row r="69">
@@ -2950,13 +2950,13 @@
         <v>16</v>
       </c>
       <c r="J69" t="n">
-        <v>-81.22</v>
+        <v>-93.52</v>
       </c>
       <c r="K69" t="n">
-        <v>352.93</v>
+        <v>406.39</v>
       </c>
       <c r="L69" t="n">
-        <v>362.15</v>
+        <v>417.01</v>
       </c>
     </row>
     <row r="70">
@@ -2992,13 +2992,13 @@
         <v>16</v>
       </c>
       <c r="J70" t="n">
-        <v>35</v>
+        <v>40.23</v>
       </c>
       <c r="K70" t="n">
-        <v>238.89</v>
+        <v>274.6</v>
       </c>
       <c r="L70" t="n">
-        <v>241.44</v>
+        <v>277.53</v>
       </c>
     </row>
     <row r="71">
@@ -3034,13 +3034,13 @@
         <v>16</v>
       </c>
       <c r="J71" t="n">
-        <v>-506.15</v>
+        <v>-587.7</v>
       </c>
       <c r="K71" t="n">
-        <v>25.63</v>
+        <v>29.76</v>
       </c>
       <c r="L71" t="n">
-        <v>506.8</v>
+        <v>588.45</v>
       </c>
     </row>
     <row r="72">
@@ -3076,13 +3076,13 @@
         <v>16</v>
       </c>
       <c r="J72" t="n">
-        <v>397.62</v>
+        <v>461.52</v>
       </c>
       <c r="K72" t="n">
-        <v>-24.1</v>
+        <v>-27.97</v>
       </c>
       <c r="L72" t="n">
-        <v>398.35</v>
+        <v>462.36</v>
       </c>
     </row>
     <row r="73">
@@ -3118,13 +3118,13 @@
         <v>17</v>
       </c>
       <c r="J73" t="n">
-        <v>-302.77</v>
+        <v>-348.31</v>
       </c>
       <c r="K73" t="n">
-        <v>-421.14</v>
+        <v>-484.5</v>
       </c>
       <c r="L73" t="n">
-        <v>518.6799999999999</v>
+        <v>596.71</v>
       </c>
     </row>
     <row r="74">
@@ -3160,13 +3160,13 @@
         <v>18</v>
       </c>
       <c r="J74" t="n">
-        <v>-22.88</v>
+        <v>-25.09</v>
       </c>
       <c r="K74" t="n">
-        <v>81.31999999999999</v>
+        <v>89.17</v>
       </c>
       <c r="L74" t="n">
-        <v>84.48</v>
+        <v>92.63</v>
       </c>
     </row>
     <row r="75">
@@ -3202,13 +3202,13 @@
         <v>16</v>
       </c>
       <c r="J75" t="n">
-        <v>85.19</v>
+        <v>96.29000000000001</v>
       </c>
       <c r="K75" t="n">
-        <v>-23.32</v>
+        <v>-26.36</v>
       </c>
       <c r="L75" t="n">
-        <v>88.31999999999999</v>
+        <v>99.83</v>
       </c>
     </row>
     <row r="76">
@@ -3244,13 +3244,13 @@
         <v>16</v>
       </c>
       <c r="J76" t="n">
-        <v>-27.87</v>
+        <v>-31.44</v>
       </c>
       <c r="K76" t="n">
-        <v>73.73999999999999</v>
+        <v>83.17</v>
       </c>
       <c r="L76" t="n">
-        <v>78.83</v>
+        <v>88.92</v>
       </c>
     </row>
     <row r="77">
@@ -3286,13 +3286,13 @@
         <v>16</v>
       </c>
       <c r="J77" t="n">
-        <v>84.59999999999999</v>
+        <v>94.58</v>
       </c>
       <c r="K77" t="n">
-        <v>-59.61</v>
+        <v>-66.64</v>
       </c>
       <c r="L77" t="n">
-        <v>103.49</v>
+        <v>115.7</v>
       </c>
     </row>
     <row r="78">
@@ -3328,13 +3328,13 @@
         <v>16</v>
       </c>
       <c r="J78" t="n">
-        <v>124.63</v>
+        <v>140.59</v>
       </c>
       <c r="K78" t="n">
-        <v>12.98</v>
+        <v>14.64</v>
       </c>
       <c r="L78" t="n">
-        <v>125.3</v>
+        <v>141.35</v>
       </c>
     </row>
     <row r="79">
@@ -3370,13 +3370,13 @@
         <v>19</v>
       </c>
       <c r="J79" t="n">
-        <v>73.26000000000001</v>
+        <v>77.55</v>
       </c>
       <c r="K79" t="n">
-        <v>3.76</v>
+        <v>3.98</v>
       </c>
       <c r="L79" t="n">
-        <v>73.36</v>
+        <v>77.65000000000001</v>
       </c>
     </row>
     <row r="80">
@@ -3412,13 +3412,13 @@
         <v>17</v>
       </c>
       <c r="J80" t="n">
-        <v>-254.6</v>
+        <v>-284.48</v>
       </c>
       <c r="K80" t="n">
-        <v>-35.71</v>
+        <v>-39.9</v>
       </c>
       <c r="L80" t="n">
-        <v>257.09</v>
+        <v>287.26</v>
       </c>
     </row>
     <row r="81">
@@ -3454,13 +3454,13 @@
         <v>19</v>
       </c>
       <c r="J81" t="n">
-        <v>-128.76</v>
+        <v>-139.83</v>
       </c>
       <c r="K81" t="n">
-        <v>205.81</v>
+        <v>223.5</v>
       </c>
       <c r="L81" t="n">
-        <v>242.77</v>
+        <v>263.63</v>
       </c>
     </row>
     <row r="82">
@@ -3496,13 +3496,13 @@
         <v>18</v>
       </c>
       <c r="J82" t="n">
-        <v>204.99</v>
+        <v>225.85</v>
       </c>
       <c r="K82" t="n">
-        <v>44.03</v>
+        <v>48.51</v>
       </c>
       <c r="L82" t="n">
-        <v>209.66</v>
+        <v>231</v>
       </c>
     </row>
     <row r="83">
@@ -3538,13 +3538,13 @@
         <v>18</v>
       </c>
       <c r="J83" t="n">
-        <v>299.11</v>
+        <v>334.9</v>
       </c>
       <c r="K83" t="n">
-        <v>237.66</v>
+        <v>266.1</v>
       </c>
       <c r="L83" t="n">
-        <v>382.03</v>
+        <v>427.74</v>
       </c>
     </row>
     <row r="84">
@@ -3580,13 +3580,13 @@
         <v>16</v>
       </c>
       <c r="J84" t="n">
-        <v>181.85</v>
+        <v>209.37</v>
       </c>
       <c r="K84" t="n">
-        <v>-176.71</v>
+        <v>-203.45</v>
       </c>
       <c r="L84" t="n">
-        <v>253.57</v>
+        <v>291.94</v>
       </c>
     </row>
     <row r="85">
@@ -3622,13 +3622,13 @@
         <v>17</v>
       </c>
       <c r="J85" t="n">
-        <v>-51.56</v>
+        <v>-58.48</v>
       </c>
       <c r="K85" t="n">
-        <v>-297.24</v>
+        <v>-337.17</v>
       </c>
       <c r="L85" t="n">
-        <v>301.68</v>
+        <v>342.21</v>
       </c>
     </row>
     <row r="86">
@@ -3664,13 +3664,13 @@
         <v>17</v>
       </c>
       <c r="J86" t="n">
-        <v>-109.47</v>
+        <v>-125.56</v>
       </c>
       <c r="K86" t="n">
-        <v>357.46</v>
+        <v>410</v>
       </c>
       <c r="L86" t="n">
-        <v>373.85</v>
+        <v>428.79</v>
       </c>
     </row>
     <row r="87">
@@ -3706,13 +3706,13 @@
         <v>17</v>
       </c>
       <c r="J87" t="n">
-        <v>464.78</v>
+        <v>534.09</v>
       </c>
       <c r="K87" t="n">
-        <v>266.55</v>
+        <v>306.3</v>
       </c>
       <c r="L87" t="n">
-        <v>535.79</v>
+        <v>615.6799999999999</v>
       </c>
     </row>
     <row r="88">
@@ -3748,13 +3748,13 @@
         <v>17</v>
       </c>
       <c r="J88" t="n">
-        <v>102.32</v>
+        <v>117.36</v>
       </c>
       <c r="K88" t="n">
-        <v>-411.91</v>
+        <v>-472.47</v>
       </c>
       <c r="L88" t="n">
-        <v>424.43</v>
+        <v>486.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
before big edit by agent
</commit_message>
<xml_diff>
--- a/output/2024-04-01.xlsx
+++ b/output/2024-04-01.xlsx
@@ -640,13 +640,13 @@
         <v>16</v>
       </c>
       <c r="J14" t="n">
-        <v>-24.82</v>
+        <v>-30.91</v>
       </c>
       <c r="K14" t="n">
-        <v>-59.45</v>
+        <v>-74.05</v>
       </c>
       <c r="L14" t="n">
-        <v>64.42</v>
+        <v>80.25</v>
       </c>
     </row>
     <row r="15">
@@ -682,13 +682,13 @@
         <v>16</v>
       </c>
       <c r="J15" t="n">
-        <v>-30.26</v>
+        <v>-38.36</v>
       </c>
       <c r="K15" t="n">
-        <v>53.17</v>
+        <v>67.38</v>
       </c>
       <c r="L15" t="n">
-        <v>61.18</v>
+        <v>77.53</v>
       </c>
     </row>
     <row r="16">
@@ -724,13 +724,13 @@
         <v>16</v>
       </c>
       <c r="J16" t="n">
-        <v>-77</v>
+        <v>-87.20999999999999</v>
       </c>
       <c r="K16" t="n">
-        <v>-58.2</v>
+        <v>-65.92</v>
       </c>
       <c r="L16" t="n">
-        <v>96.52</v>
+        <v>109.32</v>
       </c>
     </row>
     <row r="17">
@@ -766,13 +766,13 @@
         <v>16</v>
       </c>
       <c r="J17" t="n">
-        <v>41.64</v>
+        <v>48.05</v>
       </c>
       <c r="K17" t="n">
-        <v>99.48999999999999</v>
+        <v>114.8</v>
       </c>
       <c r="L17" t="n">
-        <v>107.85</v>
+        <v>124.45</v>
       </c>
     </row>
     <row r="18">
@@ -808,13 +808,13 @@
         <v>18</v>
       </c>
       <c r="J18" t="n">
-        <v>16.86</v>
+        <v>21.65</v>
       </c>
       <c r="K18" t="n">
-        <v>34.91</v>
+        <v>44.83</v>
       </c>
       <c r="L18" t="n">
-        <v>38.77</v>
+        <v>49.78</v>
       </c>
     </row>
     <row r="19">
@@ -850,13 +850,13 @@
         <v>16</v>
       </c>
       <c r="J19" t="n">
-        <v>100.79</v>
+        <v>121.95</v>
       </c>
       <c r="K19" t="n">
-        <v>-66.36</v>
+        <v>-80.29000000000001</v>
       </c>
       <c r="L19" t="n">
-        <v>120.68</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20">
@@ -892,13 +892,13 @@
         <v>19</v>
       </c>
       <c r="J20" t="n">
-        <v>141.51</v>
+        <v>174.51</v>
       </c>
       <c r="K20" t="n">
-        <v>-25.59</v>
+        <v>-31.55</v>
       </c>
       <c r="L20" t="n">
-        <v>143.81</v>
+        <v>177.34</v>
       </c>
     </row>
     <row r="21">
@@ -934,13 +934,13 @@
         <v>16</v>
       </c>
       <c r="J21" t="n">
-        <v>-136.74</v>
+        <v>-165.76</v>
       </c>
       <c r="K21" t="n">
-        <v>-54.85</v>
+        <v>-66.48999999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>147.33</v>
+        <v>178.6</v>
       </c>
     </row>
     <row r="22">
@@ -976,13 +976,13 @@
         <v>16</v>
       </c>
       <c r="J22" t="n">
-        <v>-101.54</v>
+        <v>-137.4</v>
       </c>
       <c r="K22" t="n">
-        <v>-67.16</v>
+        <v>-90.88</v>
       </c>
       <c r="L22" t="n">
-        <v>121.75</v>
+        <v>164.73</v>
       </c>
     </row>
     <row r="23">
@@ -1018,13 +1018,13 @@
         <v>16</v>
       </c>
       <c r="J23" t="n">
-        <v>135.51</v>
+        <v>198.34</v>
       </c>
       <c r="K23" t="n">
-        <v>-47.55</v>
+        <v>-69.59999999999999</v>
       </c>
       <c r="L23" t="n">
-        <v>143.61</v>
+        <v>210.2</v>
       </c>
     </row>
     <row r="24">
@@ -1060,13 +1060,13 @@
         <v>16</v>
       </c>
       <c r="J24" t="n">
-        <v>74.58</v>
+        <v>102.01</v>
       </c>
       <c r="K24" t="n">
-        <v>-189.03</v>
+        <v>-258.57</v>
       </c>
       <c r="L24" t="n">
-        <v>203.21</v>
+        <v>277.96</v>
       </c>
     </row>
     <row r="25">
@@ -1102,13 +1102,13 @@
         <v>16</v>
       </c>
       <c r="J25" t="n">
-        <v>-174.69</v>
+        <v>-222.76</v>
       </c>
       <c r="K25" t="n">
-        <v>-101.42</v>
+        <v>-129.34</v>
       </c>
       <c r="L25" t="n">
-        <v>201.99</v>
+        <v>257.59</v>
       </c>
     </row>
     <row r="26">
@@ -1144,13 +1144,13 @@
         <v>16</v>
       </c>
       <c r="J26" t="n">
-        <v>277.5</v>
+        <v>348.26</v>
       </c>
       <c r="K26" t="n">
-        <v>-537.2</v>
+        <v>-674.1799999999999</v>
       </c>
       <c r="L26" t="n">
-        <v>604.64</v>
+        <v>758.8099999999999</v>
       </c>
     </row>
     <row r="27">
@@ -1186,13 +1186,13 @@
         <v>16</v>
       </c>
       <c r="J27" t="n">
-        <v>-362.23</v>
+        <v>-484.89</v>
       </c>
       <c r="K27" t="n">
-        <v>152.88</v>
+        <v>204.65</v>
       </c>
       <c r="L27" t="n">
-        <v>393.17</v>
+        <v>526.3099999999999</v>
       </c>
     </row>
     <row r="28">
@@ -1228,13 +1228,13 @@
         <v>16</v>
       </c>
       <c r="J28" t="n">
-        <v>374.26</v>
+        <v>489.26</v>
       </c>
       <c r="K28" t="n">
-        <v>205.79</v>
+        <v>269.03</v>
       </c>
       <c r="L28" t="n">
-        <v>427.11</v>
+        <v>558.35</v>
       </c>
     </row>
     <row r="29">
@@ -1270,13 +1270,13 @@
         <v>16</v>
       </c>
       <c r="J29" t="n">
-        <v>60.12</v>
+        <v>67.86</v>
       </c>
       <c r="K29" t="n">
-        <v>-74.01000000000001</v>
+        <v>-83.54000000000001</v>
       </c>
       <c r="L29" t="n">
-        <v>95.34999999999999</v>
+        <v>107.63</v>
       </c>
     </row>
     <row r="30">
@@ -1312,13 +1312,13 @@
         <v>17</v>
       </c>
       <c r="J30" t="n">
-        <v>40.7</v>
+        <v>45.2</v>
       </c>
       <c r="K30" t="n">
-        <v>-90.86</v>
+        <v>-100.92</v>
       </c>
       <c r="L30" t="n">
-        <v>99.56</v>
+        <v>110.58</v>
       </c>
     </row>
     <row r="31">
@@ -1354,13 +1354,13 @@
         <v>16</v>
       </c>
       <c r="J31" t="n">
-        <v>1.79</v>
+        <v>2.07</v>
       </c>
       <c r="K31" t="n">
-        <v>-85.89</v>
+        <v>-99.34999999999999</v>
       </c>
       <c r="L31" t="n">
-        <v>85.91</v>
+        <v>99.37</v>
       </c>
     </row>
     <row r="32">
@@ -1396,13 +1396,13 @@
         <v>18</v>
       </c>
       <c r="J32" t="n">
-        <v>66.25</v>
+        <v>85.62</v>
       </c>
       <c r="K32" t="n">
-        <v>3.77</v>
+        <v>4.88</v>
       </c>
       <c r="L32" t="n">
-        <v>66.34999999999999</v>
+        <v>85.76000000000001</v>
       </c>
     </row>
     <row r="33">
@@ -1438,13 +1438,13 @@
         <v>16</v>
       </c>
       <c r="J33" t="n">
-        <v>37.6</v>
+        <v>45.55</v>
       </c>
       <c r="K33" t="n">
-        <v>82.64</v>
+        <v>100.13</v>
       </c>
       <c r="L33" t="n">
-        <v>90.79000000000001</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34">
@@ -1480,13 +1480,13 @@
         <v>17</v>
       </c>
       <c r="J34" t="n">
-        <v>-86.54000000000001</v>
+        <v>-104.68</v>
       </c>
       <c r="K34" t="n">
-        <v>-20.39</v>
+        <v>-24.66</v>
       </c>
       <c r="L34" t="n">
-        <v>88.91</v>
+        <v>107.55</v>
       </c>
     </row>
     <row r="35">
@@ -1522,13 +1522,13 @@
         <v>16</v>
       </c>
       <c r="J35" t="n">
-        <v>-139.35</v>
+        <v>-180.32</v>
       </c>
       <c r="K35" t="n">
-        <v>13.71</v>
+        <v>17.74</v>
       </c>
       <c r="L35" t="n">
-        <v>140.02</v>
+        <v>181.19</v>
       </c>
     </row>
     <row r="36">
@@ -1564,13 +1564,13 @@
         <v>19</v>
       </c>
       <c r="J36" t="n">
-        <v>224.92</v>
+        <v>265.89</v>
       </c>
       <c r="K36" t="n">
-        <v>-32.57</v>
+        <v>-38.51</v>
       </c>
       <c r="L36" t="n">
-        <v>227.27</v>
+        <v>268.67</v>
       </c>
     </row>
     <row r="37">
@@ -1606,13 +1606,13 @@
         <v>16</v>
       </c>
       <c r="J37" t="n">
-        <v>-156.68</v>
+        <v>-183.99</v>
       </c>
       <c r="K37" t="n">
-        <v>-85.89</v>
+        <v>-100.86</v>
       </c>
       <c r="L37" t="n">
-        <v>178.68</v>
+        <v>209.83</v>
       </c>
     </row>
     <row r="38">
@@ -1648,13 +1648,13 @@
         <v>17</v>
       </c>
       <c r="J38" t="n">
-        <v>-153.76</v>
+        <v>-223.86</v>
       </c>
       <c r="K38" t="n">
-        <v>91.18000000000001</v>
+        <v>132.75</v>
       </c>
       <c r="L38" t="n">
-        <v>178.76</v>
+        <v>260.26</v>
       </c>
     </row>
     <row r="39">
@@ -1690,13 +1690,13 @@
         <v>16</v>
       </c>
       <c r="J39" t="n">
-        <v>-189.94</v>
+        <v>-267.93</v>
       </c>
       <c r="K39" t="n">
-        <v>-94.67</v>
+        <v>-133.54</v>
       </c>
       <c r="L39" t="n">
-        <v>212.22</v>
+        <v>299.36</v>
       </c>
     </row>
     <row r="40">
@@ -1732,13 +1732,13 @@
         <v>17</v>
       </c>
       <c r="J40" t="n">
-        <v>120.46</v>
+        <v>151.92</v>
       </c>
       <c r="K40" t="n">
-        <v>-329.29</v>
+        <v>-415.3</v>
       </c>
       <c r="L40" t="n">
-        <v>350.63</v>
+        <v>442.21</v>
       </c>
     </row>
     <row r="41">
@@ -1774,13 +1774,13 @@
         <v>16</v>
       </c>
       <c r="J41" t="n">
-        <v>241.84</v>
+        <v>323.71</v>
       </c>
       <c r="K41" t="n">
-        <v>256.71</v>
+        <v>343.61</v>
       </c>
       <c r="L41" t="n">
-        <v>352.68</v>
+        <v>472.08</v>
       </c>
     </row>
     <row r="42">
@@ -1816,13 +1816,13 @@
         <v>18</v>
       </c>
       <c r="J42" t="n">
-        <v>-155.81</v>
+        <v>-207.33</v>
       </c>
       <c r="K42" t="n">
-        <v>-402.73</v>
+        <v>-535.89</v>
       </c>
       <c r="L42" t="n">
-        <v>431.81</v>
+        <v>574.6</v>
       </c>
     </row>
     <row r="43">
@@ -1858,13 +1858,13 @@
         <v>16</v>
       </c>
       <c r="J43" t="n">
-        <v>218.77</v>
+        <v>323.01</v>
       </c>
       <c r="K43" t="n">
-        <v>-159.88</v>
+        <v>-236.05</v>
       </c>
       <c r="L43" t="n">
-        <v>270.96</v>
+        <v>400.07</v>
       </c>
     </row>
     <row r="44">
@@ -1900,13 +1900,13 @@
         <v>17</v>
       </c>
       <c r="J44" t="n">
-        <v>53.17</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="K44" t="n">
-        <v>-27.62</v>
+        <v>-34.14</v>
       </c>
       <c r="L44" t="n">
-        <v>59.92</v>
+        <v>74.05</v>
       </c>
     </row>
     <row r="45">
@@ -1942,13 +1942,13 @@
         <v>16</v>
       </c>
       <c r="J45" t="n">
-        <v>79.44</v>
+        <v>92.05</v>
       </c>
       <c r="K45" t="n">
-        <v>24.47</v>
+        <v>28.36</v>
       </c>
       <c r="L45" t="n">
-        <v>83.12</v>
+        <v>96.31999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -1984,13 +1984,13 @@
         <v>19</v>
       </c>
       <c r="J46" t="n">
-        <v>65.34</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="K46" t="n">
-        <v>-54.17</v>
+        <v>-61.97</v>
       </c>
       <c r="L46" t="n">
-        <v>84.87</v>
+        <v>97.08</v>
       </c>
     </row>
     <row r="47">
@@ -2026,13 +2026,13 @@
         <v>19</v>
       </c>
       <c r="J47" t="n">
-        <v>-59.9</v>
+        <v>-75.93000000000001</v>
       </c>
       <c r="K47" t="n">
-        <v>-47.59</v>
+        <v>-60.32</v>
       </c>
       <c r="L47" t="n">
-        <v>76.51000000000001</v>
+        <v>96.98</v>
       </c>
     </row>
     <row r="48">
@@ -2068,13 +2068,13 @@
         <v>16</v>
       </c>
       <c r="J48" t="n">
-        <v>26.7</v>
+        <v>35.13</v>
       </c>
       <c r="K48" t="n">
-        <v>83.65000000000001</v>
+        <v>110.07</v>
       </c>
       <c r="L48" t="n">
-        <v>87.8</v>
+        <v>115.54</v>
       </c>
     </row>
     <row r="49">
@@ -2110,13 +2110,13 @@
         <v>16</v>
       </c>
       <c r="J49" t="n">
-        <v>9.41</v>
+        <v>11.87</v>
       </c>
       <c r="K49" t="n">
-        <v>77.55</v>
+        <v>97.81999999999999</v>
       </c>
       <c r="L49" t="n">
-        <v>78.12</v>
+        <v>98.54000000000001</v>
       </c>
     </row>
     <row r="50">
@@ -2152,13 +2152,13 @@
         <v>16</v>
       </c>
       <c r="J50" t="n">
-        <v>106</v>
+        <v>138.56</v>
       </c>
       <c r="K50" t="n">
-        <v>96.5</v>
+        <v>126.15</v>
       </c>
       <c r="L50" t="n">
-        <v>143.35</v>
+        <v>187.38</v>
       </c>
     </row>
     <row r="51">
@@ -2194,13 +2194,13 @@
         <v>16</v>
       </c>
       <c r="J51" t="n">
-        <v>-37.86</v>
+        <v>-45.4</v>
       </c>
       <c r="K51" t="n">
-        <v>-234.83</v>
+        <v>-281.57</v>
       </c>
       <c r="L51" t="n">
-        <v>237.87</v>
+        <v>285.21</v>
       </c>
     </row>
     <row r="52">
@@ -2236,13 +2236,13 @@
         <v>16</v>
       </c>
       <c r="J52" t="n">
-        <v>-49.28</v>
+        <v>-57.03</v>
       </c>
       <c r="K52" t="n">
-        <v>209.19</v>
+        <v>242.07</v>
       </c>
       <c r="L52" t="n">
-        <v>214.92</v>
+        <v>248.69</v>
       </c>
     </row>
     <row r="53">
@@ -2278,13 +2278,13 @@
         <v>18</v>
       </c>
       <c r="J53" t="n">
-        <v>199.97</v>
+        <v>281.22</v>
       </c>
       <c r="K53" t="n">
-        <v>37.17</v>
+        <v>52.27</v>
       </c>
       <c r="L53" t="n">
-        <v>203.39</v>
+        <v>286.04</v>
       </c>
     </row>
     <row r="54">
@@ -2320,13 +2320,13 @@
         <v>17</v>
       </c>
       <c r="J54" t="n">
-        <v>249.82</v>
+        <v>339.63</v>
       </c>
       <c r="K54" t="n">
-        <v>-75.67</v>
+        <v>-102.87</v>
       </c>
       <c r="L54" t="n">
-        <v>261.03</v>
+        <v>354.86</v>
       </c>
     </row>
     <row r="55">
@@ -2362,13 +2362,13 @@
         <v>16</v>
       </c>
       <c r="J55" t="n">
-        <v>-222.15</v>
+        <v>-307.21</v>
       </c>
       <c r="K55" t="n">
-        <v>-151.44</v>
+        <v>-209.43</v>
       </c>
       <c r="L55" t="n">
-        <v>268.86</v>
+        <v>371.81</v>
       </c>
     </row>
     <row r="56">
@@ -2404,13 +2404,13 @@
         <v>16</v>
       </c>
       <c r="J56" t="n">
-        <v>-200.67</v>
+        <v>-267.94</v>
       </c>
       <c r="K56" t="n">
-        <v>-490.2</v>
+        <v>-654.53</v>
       </c>
       <c r="L56" t="n">
-        <v>529.6799999999999</v>
+        <v>707.25</v>
       </c>
     </row>
     <row r="57">
@@ -2446,13 +2446,13 @@
         <v>16</v>
       </c>
       <c r="J57" t="n">
-        <v>262.51</v>
+        <v>379.07</v>
       </c>
       <c r="K57" t="n">
-        <v>159.56</v>
+        <v>230.41</v>
       </c>
       <c r="L57" t="n">
-        <v>307.2</v>
+        <v>443.6</v>
       </c>
     </row>
     <row r="58">
@@ -2488,13 +2488,13 @@
         <v>17</v>
       </c>
       <c r="J58" t="n">
-        <v>-245.52</v>
+        <v>-338.07</v>
       </c>
       <c r="K58" t="n">
-        <v>-366.34</v>
+        <v>-504.43</v>
       </c>
       <c r="L58" t="n">
-        <v>441</v>
+        <v>607.24</v>
       </c>
     </row>
     <row r="59">
@@ -2530,13 +2530,13 @@
         <v>18</v>
       </c>
       <c r="J59" t="n">
-        <v>-53.58</v>
+        <v>-61.64</v>
       </c>
       <c r="K59" t="n">
-        <v>60.25</v>
+        <v>69.31999999999999</v>
       </c>
       <c r="L59" t="n">
-        <v>80.62</v>
+        <v>92.76000000000001</v>
       </c>
     </row>
     <row r="60">
@@ -2572,13 +2572,13 @@
         <v>16</v>
       </c>
       <c r="J60" t="n">
-        <v>26.41</v>
+        <v>33.23</v>
       </c>
       <c r="K60" t="n">
-        <v>-97.8</v>
+        <v>-123.03</v>
       </c>
       <c r="L60" t="n">
-        <v>101.3</v>
+        <v>127.44</v>
       </c>
     </row>
     <row r="61">
@@ -2614,13 +2614,13 @@
         <v>18</v>
       </c>
       <c r="J61" t="n">
-        <v>-81.7</v>
+        <v>-94.83</v>
       </c>
       <c r="K61" t="n">
-        <v>-23.54</v>
+        <v>-27.32</v>
       </c>
       <c r="L61" t="n">
-        <v>85.02</v>
+        <v>98.69</v>
       </c>
     </row>
     <row r="62">
@@ -2656,13 +2656,13 @@
         <v>17</v>
       </c>
       <c r="J62" t="n">
-        <v>104.5</v>
+        <v>116.92</v>
       </c>
       <c r="K62" t="n">
-        <v>-83.04000000000001</v>
+        <v>-92.91</v>
       </c>
       <c r="L62" t="n">
-        <v>133.47</v>
+        <v>149.34</v>
       </c>
     </row>
     <row r="63">
@@ -2698,13 +2698,13 @@
         <v>19</v>
       </c>
       <c r="J63" t="n">
-        <v>-51.72</v>
+        <v>-64.90000000000001</v>
       </c>
       <c r="K63" t="n">
-        <v>75.34</v>
+        <v>94.54000000000001</v>
       </c>
       <c r="L63" t="n">
-        <v>91.38</v>
+        <v>114.67</v>
       </c>
     </row>
     <row r="64">
@@ -2740,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="J64" t="n">
-        <v>-71.95999999999999</v>
+        <v>-91.83</v>
       </c>
       <c r="K64" t="n">
-        <v>53.41</v>
+        <v>68.16</v>
       </c>
       <c r="L64" t="n">
-        <v>89.61</v>
+        <v>114.36</v>
       </c>
     </row>
     <row r="65">
@@ -2782,13 +2782,13 @@
         <v>19</v>
       </c>
       <c r="J65" t="n">
-        <v>-109.8</v>
+        <v>-135.08</v>
       </c>
       <c r="K65" t="n">
-        <v>-190.61</v>
+        <v>-234.49</v>
       </c>
       <c r="L65" t="n">
-        <v>219.97</v>
+        <v>270.62</v>
       </c>
     </row>
     <row r="66">
@@ -2824,13 +2824,13 @@
         <v>16</v>
       </c>
       <c r="J66" t="n">
-        <v>51.48</v>
+        <v>67.97</v>
       </c>
       <c r="K66" t="n">
-        <v>-170.87</v>
+        <v>-225.63</v>
       </c>
       <c r="L66" t="n">
-        <v>178.46</v>
+        <v>235.64</v>
       </c>
     </row>
     <row r="67">
@@ -2866,13 +2866,13 @@
         <v>17</v>
       </c>
       <c r="J67" t="n">
-        <v>263.37</v>
+        <v>309.95</v>
       </c>
       <c r="K67" t="n">
-        <v>-56.01</v>
+        <v>-65.91</v>
       </c>
       <c r="L67" t="n">
-        <v>269.26</v>
+        <v>316.89</v>
       </c>
     </row>
     <row r="68">
@@ -2908,13 +2908,13 @@
         <v>19</v>
       </c>
       <c r="J68" t="n">
-        <v>68.98999999999999</v>
+        <v>88.36</v>
       </c>
       <c r="K68" t="n">
-        <v>-224.71</v>
+        <v>-287.82</v>
       </c>
       <c r="L68" t="n">
-        <v>235.07</v>
+        <v>301.08</v>
       </c>
     </row>
     <row r="69">
@@ -2950,13 +2950,13 @@
         <v>17</v>
       </c>
       <c r="J69" t="n">
-        <v>-206.1</v>
+        <v>-263.96</v>
       </c>
       <c r="K69" t="n">
-        <v>-310.8</v>
+        <v>-398.04</v>
       </c>
       <c r="L69" t="n">
-        <v>372.93</v>
+        <v>477.6</v>
       </c>
     </row>
     <row r="70">
@@ -2992,13 +2992,13 @@
         <v>16</v>
       </c>
       <c r="J70" t="n">
-        <v>204.59</v>
+        <v>300.71</v>
       </c>
       <c r="K70" t="n">
-        <v>41.29</v>
+        <v>60.69</v>
       </c>
       <c r="L70" t="n">
-        <v>208.72</v>
+        <v>306.77</v>
       </c>
     </row>
     <row r="71">
@@ -3034,13 +3034,13 @@
         <v>19</v>
       </c>
       <c r="J71" t="n">
-        <v>-184.79</v>
+        <v>-278.4</v>
       </c>
       <c r="K71" t="n">
-        <v>-197.29</v>
+        <v>-297.24</v>
       </c>
       <c r="L71" t="n">
-        <v>270.32</v>
+        <v>407.26</v>
       </c>
     </row>
     <row r="72">
@@ -3076,13 +3076,13 @@
         <v>16</v>
       </c>
       <c r="J72" t="n">
-        <v>88.03</v>
+        <v>124.64</v>
       </c>
       <c r="K72" t="n">
-        <v>-314.73</v>
+        <v>-445.64</v>
       </c>
       <c r="L72" t="n">
-        <v>326.8</v>
+        <v>462.74</v>
       </c>
     </row>
     <row r="73">
@@ -3118,13 +3118,13 @@
         <v>16</v>
       </c>
       <c r="J73" t="n">
-        <v>295.87</v>
+        <v>429.18</v>
       </c>
       <c r="K73" t="n">
-        <v>145.49</v>
+        <v>211.03</v>
       </c>
       <c r="L73" t="n">
-        <v>329.71</v>
+        <v>478.26</v>
       </c>
     </row>
     <row r="74">
@@ -3160,13 +3160,13 @@
         <v>16</v>
       </c>
       <c r="J74" t="n">
-        <v>-50.95</v>
+        <v>-65.61</v>
       </c>
       <c r="K74" t="n">
-        <v>-51.96</v>
+        <v>-66.91</v>
       </c>
       <c r="L74" t="n">
-        <v>72.77</v>
+        <v>93.70999999999999</v>
       </c>
     </row>
     <row r="75">
@@ -3202,13 +3202,13 @@
         <v>16</v>
       </c>
       <c r="J75" t="n">
-        <v>-64.26000000000001</v>
+        <v>-74.41</v>
       </c>
       <c r="K75" t="n">
-        <v>-63.87</v>
+        <v>-73.95</v>
       </c>
       <c r="L75" t="n">
-        <v>90.59999999999999</v>
+        <v>104.91</v>
       </c>
     </row>
     <row r="76">
@@ -3244,13 +3244,13 @@
         <v>16</v>
       </c>
       <c r="J76" t="n">
-        <v>-65.08</v>
+        <v>-74.42</v>
       </c>
       <c r="K76" t="n">
-        <v>-63.54</v>
+        <v>-72.65000000000001</v>
       </c>
       <c r="L76" t="n">
-        <v>90.95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="77">
@@ -3286,13 +3286,13 @@
         <v>16</v>
       </c>
       <c r="J77" t="n">
-        <v>-22.28</v>
+        <v>-27.33</v>
       </c>
       <c r="K77" t="n">
-        <v>-127.49</v>
+        <v>-156.4</v>
       </c>
       <c r="L77" t="n">
-        <v>129.43</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="78">
@@ -3328,13 +3328,13 @@
         <v>16</v>
       </c>
       <c r="J78" t="n">
-        <v>-129.41</v>
+        <v>-139.23</v>
       </c>
       <c r="K78" t="n">
-        <v>-88.5</v>
+        <v>-95.22</v>
       </c>
       <c r="L78" t="n">
-        <v>156.77</v>
+        <v>168.68</v>
       </c>
     </row>
     <row r="79">
@@ -3370,13 +3370,13 @@
         <v>18</v>
       </c>
       <c r="J79" t="n">
-        <v>9.73</v>
+        <v>12.46</v>
       </c>
       <c r="K79" t="n">
-        <v>75.90000000000001</v>
+        <v>97.19</v>
       </c>
       <c r="L79" t="n">
-        <v>76.53</v>
+        <v>97.98999999999999</v>
       </c>
     </row>
     <row r="80">
@@ -3412,13 +3412,13 @@
         <v>16</v>
       </c>
       <c r="J80" t="n">
-        <v>-238.13</v>
+        <v>-281.07</v>
       </c>
       <c r="K80" t="n">
-        <v>90.84999999999999</v>
+        <v>107.23</v>
       </c>
       <c r="L80" t="n">
-        <v>254.88</v>
+        <v>300.83</v>
       </c>
     </row>
     <row r="81">
@@ -3454,13 +3454,13 @@
         <v>17</v>
       </c>
       <c r="J81" t="n">
-        <v>-67.41</v>
+        <v>-86.81999999999999</v>
       </c>
       <c r="K81" t="n">
-        <v>-172.67</v>
+        <v>-222.39</v>
       </c>
       <c r="L81" t="n">
-        <v>185.36</v>
+        <v>238.73</v>
       </c>
     </row>
     <row r="82">
@@ -3496,13 +3496,13 @@
         <v>18</v>
       </c>
       <c r="J82" t="n">
-        <v>-140.23</v>
+        <v>-176.87</v>
       </c>
       <c r="K82" t="n">
-        <v>104.72</v>
+        <v>132.08</v>
       </c>
       <c r="L82" t="n">
-        <v>175.02</v>
+        <v>220.74</v>
       </c>
     </row>
     <row r="83">
@@ -3538,13 +3538,13 @@
         <v>16</v>
       </c>
       <c r="J83" t="n">
-        <v>-341.47</v>
+        <v>-452.74</v>
       </c>
       <c r="K83" t="n">
-        <v>-24.25</v>
+        <v>-32.15</v>
       </c>
       <c r="L83" t="n">
-        <v>342.33</v>
+        <v>453.88</v>
       </c>
     </row>
     <row r="84">
@@ -3580,13 +3580,13 @@
         <v>16</v>
       </c>
       <c r="J84" t="n">
-        <v>260.18</v>
+        <v>355.45</v>
       </c>
       <c r="K84" t="n">
-        <v>-35.94</v>
+        <v>-49.1</v>
       </c>
       <c r="L84" t="n">
-        <v>262.65</v>
+        <v>358.83</v>
       </c>
     </row>
     <row r="85">
@@ -3622,13 +3622,13 @@
         <v>16</v>
       </c>
       <c r="J85" t="n">
-        <v>317.32</v>
+        <v>415.74</v>
       </c>
       <c r="K85" t="n">
-        <v>119.41</v>
+        <v>156.45</v>
       </c>
       <c r="L85" t="n">
-        <v>339.04</v>
+        <v>444.2</v>
       </c>
     </row>
     <row r="86">
@@ -3664,13 +3664,13 @@
         <v>16</v>
       </c>
       <c r="J86" t="n">
-        <v>-228.41</v>
+        <v>-312.85</v>
       </c>
       <c r="K86" t="n">
-        <v>-448.38</v>
+        <v>-614.12</v>
       </c>
       <c r="L86" t="n">
-        <v>503.2</v>
+        <v>689.21</v>
       </c>
     </row>
     <row r="87">
@@ -3706,13 +3706,13 @@
         <v>19</v>
       </c>
       <c r="J87" t="n">
-        <v>-7.69</v>
+        <v>-11</v>
       </c>
       <c r="K87" t="n">
-        <v>-412.22</v>
+        <v>-589.53</v>
       </c>
       <c r="L87" t="n">
-        <v>412.29</v>
+        <v>589.63</v>
       </c>
     </row>
     <row r="88">
@@ -3748,13 +3748,13 @@
         <v>18</v>
       </c>
       <c r="J88" t="n">
-        <v>-373.51</v>
+        <v>-514.42</v>
       </c>
       <c r="K88" t="n">
-        <v>-159.12</v>
+        <v>-219.16</v>
       </c>
       <c r="L88" t="n">
-        <v>405.99</v>
+        <v>559.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
xui znaet uze v rot ebal ety dissertaciyu
</commit_message>
<xml_diff>
--- a/output/2024-04-01.xlsx
+++ b/output/2024-04-01.xlsx
@@ -640,13 +640,13 @@
         <v>16</v>
       </c>
       <c r="J14" t="n">
-        <v>-30.91</v>
+        <v>-47.57</v>
       </c>
       <c r="K14" t="n">
-        <v>-74.05</v>
+        <v>-113.95</v>
       </c>
       <c r="L14" t="n">
-        <v>80.25</v>
+        <v>123.48</v>
       </c>
     </row>
     <row r="15">
@@ -682,13 +682,13 @@
         <v>16</v>
       </c>
       <c r="J15" t="n">
-        <v>-38.36</v>
+        <v>-58.8</v>
       </c>
       <c r="K15" t="n">
-        <v>67.38</v>
+        <v>103.29</v>
       </c>
       <c r="L15" t="n">
-        <v>77.53</v>
+        <v>118.85</v>
       </c>
     </row>
     <row r="16">
@@ -724,13 +724,13 @@
         <v>16</v>
       </c>
       <c r="J16" t="n">
-        <v>-87.20999999999999</v>
+        <v>-133.44</v>
       </c>
       <c r="K16" t="n">
-        <v>-65.92</v>
+        <v>-100.87</v>
       </c>
       <c r="L16" t="n">
-        <v>109.32</v>
+        <v>167.27</v>
       </c>
     </row>
     <row r="17">
@@ -766,13 +766,13 @@
         <v>16</v>
       </c>
       <c r="J17" t="n">
-        <v>48.05</v>
+        <v>59.9</v>
       </c>
       <c r="K17" t="n">
-        <v>114.8</v>
+        <v>143.13</v>
       </c>
       <c r="L17" t="n">
-        <v>124.45</v>
+        <v>155.16</v>
       </c>
     </row>
     <row r="18">
@@ -808,13 +808,13 @@
         <v>18</v>
       </c>
       <c r="J18" t="n">
-        <v>21.65</v>
+        <v>27.37</v>
       </c>
       <c r="K18" t="n">
-        <v>44.83</v>
+        <v>56.67</v>
       </c>
       <c r="L18" t="n">
-        <v>49.78</v>
+        <v>62.94</v>
       </c>
     </row>
     <row r="19">
@@ -850,13 +850,13 @@
         <v>16</v>
       </c>
       <c r="J19" t="n">
-        <v>121.95</v>
+        <v>180.72</v>
       </c>
       <c r="K19" t="n">
-        <v>-80.29000000000001</v>
+        <v>-118.99</v>
       </c>
       <c r="L19" t="n">
-        <v>146</v>
+        <v>216.38</v>
       </c>
     </row>
     <row r="20">
@@ -1270,13 +1270,13 @@
         <v>16</v>
       </c>
       <c r="J29" t="n">
-        <v>67.86</v>
+        <v>101.1</v>
       </c>
       <c r="K29" t="n">
-        <v>-83.54000000000001</v>
+        <v>-124.46</v>
       </c>
       <c r="L29" t="n">
-        <v>107.63</v>
+        <v>160.35</v>
       </c>
     </row>
     <row r="30">
@@ -1312,13 +1312,13 @@
         <v>17</v>
       </c>
       <c r="J30" t="n">
-        <v>45.2</v>
+        <v>69.3</v>
       </c>
       <c r="K30" t="n">
-        <v>-100.92</v>
+        <v>-154.71</v>
       </c>
       <c r="L30" t="n">
-        <v>110.58</v>
+        <v>169.52</v>
       </c>
     </row>
     <row r="31">
@@ -1354,13 +1354,13 @@
         <v>16</v>
       </c>
       <c r="J31" t="n">
-        <v>2.07</v>
+        <v>2.97</v>
       </c>
       <c r="K31" t="n">
-        <v>-99.34999999999999</v>
+        <v>-142.96</v>
       </c>
       <c r="L31" t="n">
-        <v>99.37</v>
+        <v>142.99</v>
       </c>
     </row>
     <row r="32">
@@ -1396,13 +1396,13 @@
         <v>18</v>
       </c>
       <c r="J32" t="n">
-        <v>85.62</v>
+        <v>108.91</v>
       </c>
       <c r="K32" t="n">
-        <v>4.88</v>
+        <v>6.2</v>
       </c>
       <c r="L32" t="n">
-        <v>85.76000000000001</v>
+        <v>109.08</v>
       </c>
     </row>
     <row r="33">
@@ -1438,13 +1438,13 @@
         <v>16</v>
       </c>
       <c r="J33" t="n">
-        <v>45.55</v>
+        <v>61.96</v>
       </c>
       <c r="K33" t="n">
-        <v>100.13</v>
+        <v>136.18</v>
       </c>
       <c r="L33" t="n">
-        <v>110</v>
+        <v>149.62</v>
       </c>
     </row>
     <row r="34">
@@ -1480,13 +1480,13 @@
         <v>17</v>
       </c>
       <c r="J34" t="n">
-        <v>-104.68</v>
+        <v>-134.39</v>
       </c>
       <c r="K34" t="n">
-        <v>-24.66</v>
+        <v>-31.66</v>
       </c>
       <c r="L34" t="n">
-        <v>107.55</v>
+        <v>138.07</v>
       </c>
     </row>
     <row r="35">
@@ -1900,13 +1900,13 @@
         <v>17</v>
       </c>
       <c r="J44" t="n">
-        <v>65.70999999999999</v>
+        <v>86.31</v>
       </c>
       <c r="K44" t="n">
-        <v>-34.14</v>
+        <v>-44.84</v>
       </c>
       <c r="L44" t="n">
-        <v>74.05</v>
+        <v>97.26000000000001</v>
       </c>
     </row>
     <row r="45">
@@ -1942,13 +1942,13 @@
         <v>16</v>
       </c>
       <c r="J45" t="n">
-        <v>92.05</v>
+        <v>142.99</v>
       </c>
       <c r="K45" t="n">
-        <v>28.36</v>
+        <v>44.05</v>
       </c>
       <c r="L45" t="n">
-        <v>96.31999999999999</v>
+        <v>149.62</v>
       </c>
     </row>
     <row r="46">
@@ -1984,13 +1984,13 @@
         <v>19</v>
       </c>
       <c r="J46" t="n">
-        <v>74.73999999999999</v>
+        <v>112.2</v>
       </c>
       <c r="K46" t="n">
-        <v>-61.97</v>
+        <v>-93.03</v>
       </c>
       <c r="L46" t="n">
-        <v>97.08</v>
+        <v>145.75</v>
       </c>
     </row>
     <row r="47">
@@ -2026,13 +2026,13 @@
         <v>19</v>
       </c>
       <c r="J47" t="n">
-        <v>-75.93000000000001</v>
+        <v>-106.42</v>
       </c>
       <c r="K47" t="n">
-        <v>-60.32</v>
+        <v>-84.54000000000001</v>
       </c>
       <c r="L47" t="n">
-        <v>96.98</v>
+        <v>135.91</v>
       </c>
     </row>
     <row r="48">
@@ -2068,13 +2068,13 @@
         <v>16</v>
       </c>
       <c r="J48" t="n">
-        <v>35.13</v>
+        <v>54.04</v>
       </c>
       <c r="K48" t="n">
-        <v>110.07</v>
+        <v>169.33</v>
       </c>
       <c r="L48" t="n">
-        <v>115.54</v>
+        <v>177.74</v>
       </c>
     </row>
     <row r="49">
@@ -2110,13 +2110,13 @@
         <v>16</v>
       </c>
       <c r="J49" t="n">
-        <v>11.87</v>
+        <v>16.03</v>
       </c>
       <c r="K49" t="n">
-        <v>97.81999999999999</v>
+        <v>132.05</v>
       </c>
       <c r="L49" t="n">
-        <v>98.54000000000001</v>
+        <v>133.02</v>
       </c>
     </row>
     <row r="50">
@@ -2530,13 +2530,13 @@
         <v>18</v>
       </c>
       <c r="J59" t="n">
-        <v>-61.64</v>
+        <v>-88.36</v>
       </c>
       <c r="K59" t="n">
-        <v>69.31999999999999</v>
+        <v>99.36</v>
       </c>
       <c r="L59" t="n">
-        <v>92.76000000000001</v>
+        <v>132.96</v>
       </c>
     </row>
     <row r="60">
@@ -2572,13 +2572,13 @@
         <v>16</v>
       </c>
       <c r="J60" t="n">
-        <v>33.23</v>
+        <v>64.61</v>
       </c>
       <c r="K60" t="n">
-        <v>-123.03</v>
+        <v>-239.24</v>
       </c>
       <c r="L60" t="n">
-        <v>127.44</v>
+        <v>247.81</v>
       </c>
     </row>
     <row r="61">
@@ -2614,13 +2614,13 @@
         <v>18</v>
       </c>
       <c r="J61" t="n">
-        <v>-94.83</v>
+        <v>-151.75</v>
       </c>
       <c r="K61" t="n">
-        <v>-27.32</v>
+        <v>-43.72</v>
       </c>
       <c r="L61" t="n">
-        <v>98.69</v>
+        <v>157.92</v>
       </c>
     </row>
     <row r="62">
@@ -2656,13 +2656,13 @@
         <v>17</v>
       </c>
       <c r="J62" t="n">
-        <v>116.92</v>
+        <v>155.69</v>
       </c>
       <c r="K62" t="n">
-        <v>-92.91</v>
+        <v>-123.72</v>
       </c>
       <c r="L62" t="n">
-        <v>149.34</v>
+        <v>198.87</v>
       </c>
     </row>
     <row r="63">
@@ -2698,13 +2698,13 @@
         <v>19</v>
       </c>
       <c r="J63" t="n">
-        <v>-64.90000000000001</v>
+        <v>-93.54000000000001</v>
       </c>
       <c r="K63" t="n">
-        <v>94.54000000000001</v>
+        <v>136.27</v>
       </c>
       <c r="L63" t="n">
-        <v>114.67</v>
+        <v>165.29</v>
       </c>
     </row>
     <row r="64">
@@ -2740,13 +2740,13 @@
         <v>18</v>
       </c>
       <c r="J64" t="n">
-        <v>-91.83</v>
+        <v>-132.37</v>
       </c>
       <c r="K64" t="n">
-        <v>68.16</v>
+        <v>98.23999999999999</v>
       </c>
       <c r="L64" t="n">
-        <v>114.36</v>
+        <v>164.84</v>
       </c>
     </row>
     <row r="65">
@@ -3160,13 +3160,13 @@
         <v>16</v>
       </c>
       <c r="J74" t="n">
-        <v>-65.61</v>
+        <v>-117.08</v>
       </c>
       <c r="K74" t="n">
-        <v>-66.91</v>
+        <v>-119.4</v>
       </c>
       <c r="L74" t="n">
-        <v>93.70999999999999</v>
+        <v>167.22</v>
       </c>
     </row>
     <row r="75">
@@ -3202,13 +3202,13 @@
         <v>16</v>
       </c>
       <c r="J75" t="n">
-        <v>-74.41</v>
+        <v>-124.39</v>
       </c>
       <c r="K75" t="n">
-        <v>-73.95</v>
+        <v>-123.63</v>
       </c>
       <c r="L75" t="n">
-        <v>104.91</v>
+        <v>175.38</v>
       </c>
     </row>
     <row r="76">
@@ -3244,13 +3244,13 @@
         <v>16</v>
       </c>
       <c r="J76" t="n">
-        <v>-74.42</v>
+        <v>-120.19</v>
       </c>
       <c r="K76" t="n">
-        <v>-72.65000000000001</v>
+        <v>-117.34</v>
       </c>
       <c r="L76" t="n">
-        <v>104</v>
+        <v>167.97</v>
       </c>
     </row>
     <row r="77">
@@ -3286,13 +3286,13 @@
         <v>16</v>
       </c>
       <c r="J77" t="n">
-        <v>-27.33</v>
+        <v>-41.21</v>
       </c>
       <c r="K77" t="n">
-        <v>-156.4</v>
+        <v>-235.83</v>
       </c>
       <c r="L77" t="n">
-        <v>158.77</v>
+        <v>239.41</v>
       </c>
     </row>
     <row r="78">
@@ -3328,13 +3328,13 @@
         <v>16</v>
       </c>
       <c r="J78" t="n">
-        <v>-139.23</v>
+        <v>-185.69</v>
       </c>
       <c r="K78" t="n">
-        <v>-95.22</v>
+        <v>-126.99</v>
       </c>
       <c r="L78" t="n">
-        <v>168.68</v>
+        <v>224.96</v>
       </c>
     </row>
     <row r="79">
@@ -3370,13 +3370,13 @@
         <v>18</v>
       </c>
       <c r="J79" t="n">
-        <v>12.46</v>
+        <v>17.28</v>
       </c>
       <c r="K79" t="n">
-        <v>97.19</v>
+        <v>134.8</v>
       </c>
       <c r="L79" t="n">
-        <v>97.98999999999999</v>
+        <v>135.9</v>
       </c>
     </row>
     <row r="80">

</xml_diff>